<commit_message>
feat: separate urea limits for diesel+urea, default 70 L/day and 800 L/month
- Vehicle table: two urea-limit columns, enabled only for "גולדיזל + אוריאה";
  the split urea row takes these instead of the diesel limits
- Any empty daily/monthly limit (vehicle, urea, driver card, master) is sent as
  70 / 800, shown as a placeholder; monthly limit no longer required for driver/master
- Excel template + import: optional urea-limit columns, instructions updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/order-template.xlsx
+++ b/order-template.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -485,29 +485,43 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>4. אין לשנות את שורת הכותרות ואין להוסיף עמודות.</t>
+          <t xml:space="preserve">   הגבלה ריקה = 70 ליטר ליום ו-800 ליטר לחודש.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>5. שומרים את הקובץ ומעלים אותו בטופס, במסך «דלקן / כרטיס רכב».</t>
+          <t xml:space="preserve">   הגבלת אוריאה ממלאים רק כשסוג הדלק «גולדיזל + אוריאה».</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr"/>
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>4. אין לשנות את שורת הכותרות ואין להוסיף עמודות.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
+          <t>5. שומרים את הקובץ ומעלים אותו בטופס, במסך «דלקן / כרטיס רכב».</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
           <t>הזמנה עם יותר מ-10 רכבים, או עם כמה סוגי אמצעי תדלוק,</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>תפוצל אוטומטית לכמה טפסים. כל טופס יישלח לחתימה בנפרד.</t>
         </is>
@@ -524,7 +538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L301"/>
+  <dimension ref="A1:N301"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -539,6 +553,8 @@
     <col width="18" customWidth="1" min="10" max="10"/>
     <col width="18" customWidth="1" min="11" max="11"/>
     <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -579,25 +595,35 @@
       </c>
       <c r="H1" s="4" t="inlineStr">
         <is>
+          <t>הגבלת אוריאה ליום</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>הגבלת אוריאה לחודש</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
           <t>דגם רכב</t>
         </is>
       </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="K1" s="4" t="inlineStr">
         <is>
           <t>שנת יצור</t>
         </is>
       </c>
-      <c r="J1" s="4" t="inlineStr">
+      <c r="L1" s="4" t="inlineStr">
         <is>
           <t>שם נהג</t>
         </is>
       </c>
-      <c r="K1" s="4" t="inlineStr">
+      <c r="M1" s="4" t="inlineStr">
         <is>
           <t>קוד / שם מחלקה</t>
         </is>
       </c>
-      <c r="L1" s="4" t="inlineStr">
+      <c r="N1" s="4" t="inlineStr">
         <is>
           <t>שטיפומט</t>
         </is>
@@ -606,1502 +632,1502 @@
     <row r="2">
       <c r="B2" s="5" t="n"/>
       <c r="C2" s="5" t="n"/>
-      <c r="I2" s="5" t="n"/>
+      <c r="K2" s="5" t="n"/>
     </row>
     <row r="3">
       <c r="B3" s="5" t="n"/>
       <c r="C3" s="5" t="n"/>
-      <c r="I3" s="5" t="n"/>
+      <c r="K3" s="5" t="n"/>
     </row>
     <row r="4">
       <c r="B4" s="5" t="n"/>
       <c r="C4" s="5" t="n"/>
-      <c r="I4" s="5" t="n"/>
+      <c r="K4" s="5" t="n"/>
     </row>
     <row r="5">
       <c r="B5" s="5" t="n"/>
       <c r="C5" s="5" t="n"/>
-      <c r="I5" s="5" t="n"/>
+      <c r="K5" s="5" t="n"/>
     </row>
     <row r="6">
       <c r="B6" s="5" t="n"/>
       <c r="C6" s="5" t="n"/>
-      <c r="I6" s="5" t="n"/>
+      <c r="K6" s="5" t="n"/>
     </row>
     <row r="7">
       <c r="B7" s="5" t="n"/>
       <c r="C7" s="5" t="n"/>
-      <c r="I7" s="5" t="n"/>
+      <c r="K7" s="5" t="n"/>
     </row>
     <row r="8">
       <c r="B8" s="5" t="n"/>
       <c r="C8" s="5" t="n"/>
-      <c r="I8" s="5" t="n"/>
+      <c r="K8" s="5" t="n"/>
     </row>
     <row r="9">
       <c r="B9" s="5" t="n"/>
       <c r="C9" s="5" t="n"/>
-      <c r="I9" s="5" t="n"/>
+      <c r="K9" s="5" t="n"/>
     </row>
     <row r="10">
       <c r="B10" s="5" t="n"/>
       <c r="C10" s="5" t="n"/>
-      <c r="I10" s="5" t="n"/>
+      <c r="K10" s="5" t="n"/>
     </row>
     <row r="11">
       <c r="B11" s="5" t="n"/>
       <c r="C11" s="5" t="n"/>
-      <c r="I11" s="5" t="n"/>
+      <c r="K11" s="5" t="n"/>
     </row>
     <row r="12">
       <c r="B12" s="5" t="n"/>
       <c r="C12" s="5" t="n"/>
-      <c r="I12" s="5" t="n"/>
+      <c r="K12" s="5" t="n"/>
     </row>
     <row r="13">
       <c r="B13" s="5" t="n"/>
       <c r="C13" s="5" t="n"/>
-      <c r="I13" s="5" t="n"/>
+      <c r="K13" s="5" t="n"/>
     </row>
     <row r="14">
       <c r="B14" s="5" t="n"/>
       <c r="C14" s="5" t="n"/>
-      <c r="I14" s="5" t="n"/>
+      <c r="K14" s="5" t="n"/>
     </row>
     <row r="15">
       <c r="B15" s="5" t="n"/>
       <c r="C15" s="5" t="n"/>
-      <c r="I15" s="5" t="n"/>
+      <c r="K15" s="5" t="n"/>
     </row>
     <row r="16">
       <c r="B16" s="5" t="n"/>
       <c r="C16" s="5" t="n"/>
-      <c r="I16" s="5" t="n"/>
+      <c r="K16" s="5" t="n"/>
     </row>
     <row r="17">
       <c r="B17" s="5" t="n"/>
       <c r="C17" s="5" t="n"/>
-      <c r="I17" s="5" t="n"/>
+      <c r="K17" s="5" t="n"/>
     </row>
     <row r="18">
       <c r="B18" s="5" t="n"/>
       <c r="C18" s="5" t="n"/>
-      <c r="I18" s="5" t="n"/>
+      <c r="K18" s="5" t="n"/>
     </row>
     <row r="19">
       <c r="B19" s="5" t="n"/>
       <c r="C19" s="5" t="n"/>
-      <c r="I19" s="5" t="n"/>
+      <c r="K19" s="5" t="n"/>
     </row>
     <row r="20">
       <c r="B20" s="5" t="n"/>
       <c r="C20" s="5" t="n"/>
-      <c r="I20" s="5" t="n"/>
+      <c r="K20" s="5" t="n"/>
     </row>
     <row r="21">
       <c r="B21" s="5" t="n"/>
       <c r="C21" s="5" t="n"/>
-      <c r="I21" s="5" t="n"/>
+      <c r="K21" s="5" t="n"/>
     </row>
     <row r="22">
       <c r="B22" s="5" t="n"/>
       <c r="C22" s="5" t="n"/>
-      <c r="I22" s="5" t="n"/>
+      <c r="K22" s="5" t="n"/>
     </row>
     <row r="23">
       <c r="B23" s="5" t="n"/>
       <c r="C23" s="5" t="n"/>
-      <c r="I23" s="5" t="n"/>
+      <c r="K23" s="5" t="n"/>
     </row>
     <row r="24">
       <c r="B24" s="5" t="n"/>
       <c r="C24" s="5" t="n"/>
-      <c r="I24" s="5" t="n"/>
+      <c r="K24" s="5" t="n"/>
     </row>
     <row r="25">
       <c r="B25" s="5" t="n"/>
       <c r="C25" s="5" t="n"/>
-      <c r="I25" s="5" t="n"/>
+      <c r="K25" s="5" t="n"/>
     </row>
     <row r="26">
       <c r="B26" s="5" t="n"/>
       <c r="C26" s="5" t="n"/>
-      <c r="I26" s="5" t="n"/>
+      <c r="K26" s="5" t="n"/>
     </row>
     <row r="27">
       <c r="B27" s="5" t="n"/>
       <c r="C27" s="5" t="n"/>
-      <c r="I27" s="5" t="n"/>
+      <c r="K27" s="5" t="n"/>
     </row>
     <row r="28">
       <c r="B28" s="5" t="n"/>
       <c r="C28" s="5" t="n"/>
-      <c r="I28" s="5" t="n"/>
+      <c r="K28" s="5" t="n"/>
     </row>
     <row r="29">
       <c r="B29" s="5" t="n"/>
       <c r="C29" s="5" t="n"/>
-      <c r="I29" s="5" t="n"/>
+      <c r="K29" s="5" t="n"/>
     </row>
     <row r="30">
       <c r="B30" s="5" t="n"/>
       <c r="C30" s="5" t="n"/>
-      <c r="I30" s="5" t="n"/>
+      <c r="K30" s="5" t="n"/>
     </row>
     <row r="31">
       <c r="B31" s="5" t="n"/>
       <c r="C31" s="5" t="n"/>
-      <c r="I31" s="5" t="n"/>
+      <c r="K31" s="5" t="n"/>
     </row>
     <row r="32">
       <c r="B32" s="5" t="n"/>
       <c r="C32" s="5" t="n"/>
-      <c r="I32" s="5" t="n"/>
+      <c r="K32" s="5" t="n"/>
     </row>
     <row r="33">
       <c r="B33" s="5" t="n"/>
       <c r="C33" s="5" t="n"/>
-      <c r="I33" s="5" t="n"/>
+      <c r="K33" s="5" t="n"/>
     </row>
     <row r="34">
       <c r="B34" s="5" t="n"/>
       <c r="C34" s="5" t="n"/>
-      <c r="I34" s="5" t="n"/>
+      <c r="K34" s="5" t="n"/>
     </row>
     <row r="35">
       <c r="B35" s="5" t="n"/>
       <c r="C35" s="5" t="n"/>
-      <c r="I35" s="5" t="n"/>
+      <c r="K35" s="5" t="n"/>
     </row>
     <row r="36">
       <c r="B36" s="5" t="n"/>
       <c r="C36" s="5" t="n"/>
-      <c r="I36" s="5" t="n"/>
+      <c r="K36" s="5" t="n"/>
     </row>
     <row r="37">
       <c r="B37" s="5" t="n"/>
       <c r="C37" s="5" t="n"/>
-      <c r="I37" s="5" t="n"/>
+      <c r="K37" s="5" t="n"/>
     </row>
     <row r="38">
       <c r="B38" s="5" t="n"/>
       <c r="C38" s="5" t="n"/>
-      <c r="I38" s="5" t="n"/>
+      <c r="K38" s="5" t="n"/>
     </row>
     <row r="39">
       <c r="B39" s="5" t="n"/>
       <c r="C39" s="5" t="n"/>
-      <c r="I39" s="5" t="n"/>
+      <c r="K39" s="5" t="n"/>
     </row>
     <row r="40">
       <c r="B40" s="5" t="n"/>
       <c r="C40" s="5" t="n"/>
-      <c r="I40" s="5" t="n"/>
+      <c r="K40" s="5" t="n"/>
     </row>
     <row r="41">
       <c r="B41" s="5" t="n"/>
       <c r="C41" s="5" t="n"/>
-      <c r="I41" s="5" t="n"/>
+      <c r="K41" s="5" t="n"/>
     </row>
     <row r="42">
       <c r="B42" s="5" t="n"/>
       <c r="C42" s="5" t="n"/>
-      <c r="I42" s="5" t="n"/>
+      <c r="K42" s="5" t="n"/>
     </row>
     <row r="43">
       <c r="B43" s="5" t="n"/>
       <c r="C43" s="5" t="n"/>
-      <c r="I43" s="5" t="n"/>
+      <c r="K43" s="5" t="n"/>
     </row>
     <row r="44">
       <c r="B44" s="5" t="n"/>
       <c r="C44" s="5" t="n"/>
-      <c r="I44" s="5" t="n"/>
+      <c r="K44" s="5" t="n"/>
     </row>
     <row r="45">
       <c r="B45" s="5" t="n"/>
       <c r="C45" s="5" t="n"/>
-      <c r="I45" s="5" t="n"/>
+      <c r="K45" s="5" t="n"/>
     </row>
     <row r="46">
       <c r="B46" s="5" t="n"/>
       <c r="C46" s="5" t="n"/>
-      <c r="I46" s="5" t="n"/>
+      <c r="K46" s="5" t="n"/>
     </row>
     <row r="47">
       <c r="B47" s="5" t="n"/>
       <c r="C47" s="5" t="n"/>
-      <c r="I47" s="5" t="n"/>
+      <c r="K47" s="5" t="n"/>
     </row>
     <row r="48">
       <c r="B48" s="5" t="n"/>
       <c r="C48" s="5" t="n"/>
-      <c r="I48" s="5" t="n"/>
+      <c r="K48" s="5" t="n"/>
     </row>
     <row r="49">
       <c r="B49" s="5" t="n"/>
       <c r="C49" s="5" t="n"/>
-      <c r="I49" s="5" t="n"/>
+      <c r="K49" s="5" t="n"/>
     </row>
     <row r="50">
       <c r="B50" s="5" t="n"/>
       <c r="C50" s="5" t="n"/>
-      <c r="I50" s="5" t="n"/>
+      <c r="K50" s="5" t="n"/>
     </row>
     <row r="51">
       <c r="B51" s="5" t="n"/>
       <c r="C51" s="5" t="n"/>
-      <c r="I51" s="5" t="n"/>
+      <c r="K51" s="5" t="n"/>
     </row>
     <row r="52">
       <c r="B52" s="5" t="n"/>
       <c r="C52" s="5" t="n"/>
-      <c r="I52" s="5" t="n"/>
+      <c r="K52" s="5" t="n"/>
     </row>
     <row r="53">
       <c r="B53" s="5" t="n"/>
       <c r="C53" s="5" t="n"/>
-      <c r="I53" s="5" t="n"/>
+      <c r="K53" s="5" t="n"/>
     </row>
     <row r="54">
       <c r="B54" s="5" t="n"/>
       <c r="C54" s="5" t="n"/>
-      <c r="I54" s="5" t="n"/>
+      <c r="K54" s="5" t="n"/>
     </row>
     <row r="55">
       <c r="B55" s="5" t="n"/>
       <c r="C55" s="5" t="n"/>
-      <c r="I55" s="5" t="n"/>
+      <c r="K55" s="5" t="n"/>
     </row>
     <row r="56">
       <c r="B56" s="5" t="n"/>
       <c r="C56" s="5" t="n"/>
-      <c r="I56" s="5" t="n"/>
+      <c r="K56" s="5" t="n"/>
     </row>
     <row r="57">
       <c r="B57" s="5" t="n"/>
       <c r="C57" s="5" t="n"/>
-      <c r="I57" s="5" t="n"/>
+      <c r="K57" s="5" t="n"/>
     </row>
     <row r="58">
       <c r="B58" s="5" t="n"/>
       <c r="C58" s="5" t="n"/>
-      <c r="I58" s="5" t="n"/>
+      <c r="K58" s="5" t="n"/>
     </row>
     <row r="59">
       <c r="B59" s="5" t="n"/>
       <c r="C59" s="5" t="n"/>
-      <c r="I59" s="5" t="n"/>
+      <c r="K59" s="5" t="n"/>
     </row>
     <row r="60">
       <c r="B60" s="5" t="n"/>
       <c r="C60" s="5" t="n"/>
-      <c r="I60" s="5" t="n"/>
+      <c r="K60" s="5" t="n"/>
     </row>
     <row r="61">
       <c r="B61" s="5" t="n"/>
       <c r="C61" s="5" t="n"/>
-      <c r="I61" s="5" t="n"/>
+      <c r="K61" s="5" t="n"/>
     </row>
     <row r="62">
       <c r="B62" s="5" t="n"/>
       <c r="C62" s="5" t="n"/>
-      <c r="I62" s="5" t="n"/>
+      <c r="K62" s="5" t="n"/>
     </row>
     <row r="63">
       <c r="B63" s="5" t="n"/>
       <c r="C63" s="5" t="n"/>
-      <c r="I63" s="5" t="n"/>
+      <c r="K63" s="5" t="n"/>
     </row>
     <row r="64">
       <c r="B64" s="5" t="n"/>
       <c r="C64" s="5" t="n"/>
-      <c r="I64" s="5" t="n"/>
+      <c r="K64" s="5" t="n"/>
     </row>
     <row r="65">
       <c r="B65" s="5" t="n"/>
       <c r="C65" s="5" t="n"/>
-      <c r="I65" s="5" t="n"/>
+      <c r="K65" s="5" t="n"/>
     </row>
     <row r="66">
       <c r="B66" s="5" t="n"/>
       <c r="C66" s="5" t="n"/>
-      <c r="I66" s="5" t="n"/>
+      <c r="K66" s="5" t="n"/>
     </row>
     <row r="67">
       <c r="B67" s="5" t="n"/>
       <c r="C67" s="5" t="n"/>
-      <c r="I67" s="5" t="n"/>
+      <c r="K67" s="5" t="n"/>
     </row>
     <row r="68">
       <c r="B68" s="5" t="n"/>
       <c r="C68" s="5" t="n"/>
-      <c r="I68" s="5" t="n"/>
+      <c r="K68" s="5" t="n"/>
     </row>
     <row r="69">
       <c r="B69" s="5" t="n"/>
       <c r="C69" s="5" t="n"/>
-      <c r="I69" s="5" t="n"/>
+      <c r="K69" s="5" t="n"/>
     </row>
     <row r="70">
       <c r="B70" s="5" t="n"/>
       <c r="C70" s="5" t="n"/>
-      <c r="I70" s="5" t="n"/>
+      <c r="K70" s="5" t="n"/>
     </row>
     <row r="71">
       <c r="B71" s="5" t="n"/>
       <c r="C71" s="5" t="n"/>
-      <c r="I71" s="5" t="n"/>
+      <c r="K71" s="5" t="n"/>
     </row>
     <row r="72">
       <c r="B72" s="5" t="n"/>
       <c r="C72" s="5" t="n"/>
-      <c r="I72" s="5" t="n"/>
+      <c r="K72" s="5" t="n"/>
     </row>
     <row r="73">
       <c r="B73" s="5" t="n"/>
       <c r="C73" s="5" t="n"/>
-      <c r="I73" s="5" t="n"/>
+      <c r="K73" s="5" t="n"/>
     </row>
     <row r="74">
       <c r="B74" s="5" t="n"/>
       <c r="C74" s="5" t="n"/>
-      <c r="I74" s="5" t="n"/>
+      <c r="K74" s="5" t="n"/>
     </row>
     <row r="75">
       <c r="B75" s="5" t="n"/>
       <c r="C75" s="5" t="n"/>
-      <c r="I75" s="5" t="n"/>
+      <c r="K75" s="5" t="n"/>
     </row>
     <row r="76">
       <c r="B76" s="5" t="n"/>
       <c r="C76" s="5" t="n"/>
-      <c r="I76" s="5" t="n"/>
+      <c r="K76" s="5" t="n"/>
     </row>
     <row r="77">
       <c r="B77" s="5" t="n"/>
       <c r="C77" s="5" t="n"/>
-      <c r="I77" s="5" t="n"/>
+      <c r="K77" s="5" t="n"/>
     </row>
     <row r="78">
       <c r="B78" s="5" t="n"/>
       <c r="C78" s="5" t="n"/>
-      <c r="I78" s="5" t="n"/>
+      <c r="K78" s="5" t="n"/>
     </row>
     <row r="79">
       <c r="B79" s="5" t="n"/>
       <c r="C79" s="5" t="n"/>
-      <c r="I79" s="5" t="n"/>
+      <c r="K79" s="5" t="n"/>
     </row>
     <row r="80">
       <c r="B80" s="5" t="n"/>
       <c r="C80" s="5" t="n"/>
-      <c r="I80" s="5" t="n"/>
+      <c r="K80" s="5" t="n"/>
     </row>
     <row r="81">
       <c r="B81" s="5" t="n"/>
       <c r="C81" s="5" t="n"/>
-      <c r="I81" s="5" t="n"/>
+      <c r="K81" s="5" t="n"/>
     </row>
     <row r="82">
       <c r="B82" s="5" t="n"/>
       <c r="C82" s="5" t="n"/>
-      <c r="I82" s="5" t="n"/>
+      <c r="K82" s="5" t="n"/>
     </row>
     <row r="83">
       <c r="B83" s="5" t="n"/>
       <c r="C83" s="5" t="n"/>
-      <c r="I83" s="5" t="n"/>
+      <c r="K83" s="5" t="n"/>
     </row>
     <row r="84">
       <c r="B84" s="5" t="n"/>
       <c r="C84" s="5" t="n"/>
-      <c r="I84" s="5" t="n"/>
+      <c r="K84" s="5" t="n"/>
     </row>
     <row r="85">
       <c r="B85" s="5" t="n"/>
       <c r="C85" s="5" t="n"/>
-      <c r="I85" s="5" t="n"/>
+      <c r="K85" s="5" t="n"/>
     </row>
     <row r="86">
       <c r="B86" s="5" t="n"/>
       <c r="C86" s="5" t="n"/>
-      <c r="I86" s="5" t="n"/>
+      <c r="K86" s="5" t="n"/>
     </row>
     <row r="87">
       <c r="B87" s="5" t="n"/>
       <c r="C87" s="5" t="n"/>
-      <c r="I87" s="5" t="n"/>
+      <c r="K87" s="5" t="n"/>
     </row>
     <row r="88">
       <c r="B88" s="5" t="n"/>
       <c r="C88" s="5" t="n"/>
-      <c r="I88" s="5" t="n"/>
+      <c r="K88" s="5" t="n"/>
     </row>
     <row r="89">
       <c r="B89" s="5" t="n"/>
       <c r="C89" s="5" t="n"/>
-      <c r="I89" s="5" t="n"/>
+      <c r="K89" s="5" t="n"/>
     </row>
     <row r="90">
       <c r="B90" s="5" t="n"/>
       <c r="C90" s="5" t="n"/>
-      <c r="I90" s="5" t="n"/>
+      <c r="K90" s="5" t="n"/>
     </row>
     <row r="91">
       <c r="B91" s="5" t="n"/>
       <c r="C91" s="5" t="n"/>
-      <c r="I91" s="5" t="n"/>
+      <c r="K91" s="5" t="n"/>
     </row>
     <row r="92">
       <c r="B92" s="5" t="n"/>
       <c r="C92" s="5" t="n"/>
-      <c r="I92" s="5" t="n"/>
+      <c r="K92" s="5" t="n"/>
     </row>
     <row r="93">
       <c r="B93" s="5" t="n"/>
       <c r="C93" s="5" t="n"/>
-      <c r="I93" s="5" t="n"/>
+      <c r="K93" s="5" t="n"/>
     </row>
     <row r="94">
       <c r="B94" s="5" t="n"/>
       <c r="C94" s="5" t="n"/>
-      <c r="I94" s="5" t="n"/>
+      <c r="K94" s="5" t="n"/>
     </row>
     <row r="95">
       <c r="B95" s="5" t="n"/>
       <c r="C95" s="5" t="n"/>
-      <c r="I95" s="5" t="n"/>
+      <c r="K95" s="5" t="n"/>
     </row>
     <row r="96">
       <c r="B96" s="5" t="n"/>
       <c r="C96" s="5" t="n"/>
-      <c r="I96" s="5" t="n"/>
+      <c r="K96" s="5" t="n"/>
     </row>
     <row r="97">
       <c r="B97" s="5" t="n"/>
       <c r="C97" s="5" t="n"/>
-      <c r="I97" s="5" t="n"/>
+      <c r="K97" s="5" t="n"/>
     </row>
     <row r="98">
       <c r="B98" s="5" t="n"/>
       <c r="C98" s="5" t="n"/>
-      <c r="I98" s="5" t="n"/>
+      <c r="K98" s="5" t="n"/>
     </row>
     <row r="99">
       <c r="B99" s="5" t="n"/>
       <c r="C99" s="5" t="n"/>
-      <c r="I99" s="5" t="n"/>
+      <c r="K99" s="5" t="n"/>
     </row>
     <row r="100">
       <c r="B100" s="5" t="n"/>
       <c r="C100" s="5" t="n"/>
-      <c r="I100" s="5" t="n"/>
+      <c r="K100" s="5" t="n"/>
     </row>
     <row r="101">
       <c r="B101" s="5" t="n"/>
       <c r="C101" s="5" t="n"/>
-      <c r="I101" s="5" t="n"/>
+      <c r="K101" s="5" t="n"/>
     </row>
     <row r="102">
       <c r="B102" s="5" t="n"/>
       <c r="C102" s="5" t="n"/>
-      <c r="I102" s="5" t="n"/>
+      <c r="K102" s="5" t="n"/>
     </row>
     <row r="103">
       <c r="B103" s="5" t="n"/>
       <c r="C103" s="5" t="n"/>
-      <c r="I103" s="5" t="n"/>
+      <c r="K103" s="5" t="n"/>
     </row>
     <row r="104">
       <c r="B104" s="5" t="n"/>
       <c r="C104" s="5" t="n"/>
-      <c r="I104" s="5" t="n"/>
+      <c r="K104" s="5" t="n"/>
     </row>
     <row r="105">
       <c r="B105" s="5" t="n"/>
       <c r="C105" s="5" t="n"/>
-      <c r="I105" s="5" t="n"/>
+      <c r="K105" s="5" t="n"/>
     </row>
     <row r="106">
       <c r="B106" s="5" t="n"/>
       <c r="C106" s="5" t="n"/>
-      <c r="I106" s="5" t="n"/>
+      <c r="K106" s="5" t="n"/>
     </row>
     <row r="107">
       <c r="B107" s="5" t="n"/>
       <c r="C107" s="5" t="n"/>
-      <c r="I107" s="5" t="n"/>
+      <c r="K107" s="5" t="n"/>
     </row>
     <row r="108">
       <c r="B108" s="5" t="n"/>
       <c r="C108" s="5" t="n"/>
-      <c r="I108" s="5" t="n"/>
+      <c r="K108" s="5" t="n"/>
     </row>
     <row r="109">
       <c r="B109" s="5" t="n"/>
       <c r="C109" s="5" t="n"/>
-      <c r="I109" s="5" t="n"/>
+      <c r="K109" s="5" t="n"/>
     </row>
     <row r="110">
       <c r="B110" s="5" t="n"/>
       <c r="C110" s="5" t="n"/>
-      <c r="I110" s="5" t="n"/>
+      <c r="K110" s="5" t="n"/>
     </row>
     <row r="111">
       <c r="B111" s="5" t="n"/>
       <c r="C111" s="5" t="n"/>
-      <c r="I111" s="5" t="n"/>
+      <c r="K111" s="5" t="n"/>
     </row>
     <row r="112">
       <c r="B112" s="5" t="n"/>
       <c r="C112" s="5" t="n"/>
-      <c r="I112" s="5" t="n"/>
+      <c r="K112" s="5" t="n"/>
     </row>
     <row r="113">
       <c r="B113" s="5" t="n"/>
       <c r="C113" s="5" t="n"/>
-      <c r="I113" s="5" t="n"/>
+      <c r="K113" s="5" t="n"/>
     </row>
     <row r="114">
       <c r="B114" s="5" t="n"/>
       <c r="C114" s="5" t="n"/>
-      <c r="I114" s="5" t="n"/>
+      <c r="K114" s="5" t="n"/>
     </row>
     <row r="115">
       <c r="B115" s="5" t="n"/>
       <c r="C115" s="5" t="n"/>
-      <c r="I115" s="5" t="n"/>
+      <c r="K115" s="5" t="n"/>
     </row>
     <row r="116">
       <c r="B116" s="5" t="n"/>
       <c r="C116" s="5" t="n"/>
-      <c r="I116" s="5" t="n"/>
+      <c r="K116" s="5" t="n"/>
     </row>
     <row r="117">
       <c r="B117" s="5" t="n"/>
       <c r="C117" s="5" t="n"/>
-      <c r="I117" s="5" t="n"/>
+      <c r="K117" s="5" t="n"/>
     </row>
     <row r="118">
       <c r="B118" s="5" t="n"/>
       <c r="C118" s="5" t="n"/>
-      <c r="I118" s="5" t="n"/>
+      <c r="K118" s="5" t="n"/>
     </row>
     <row r="119">
       <c r="B119" s="5" t="n"/>
       <c r="C119" s="5" t="n"/>
-      <c r="I119" s="5" t="n"/>
+      <c r="K119" s="5" t="n"/>
     </row>
     <row r="120">
       <c r="B120" s="5" t="n"/>
       <c r="C120" s="5" t="n"/>
-      <c r="I120" s="5" t="n"/>
+      <c r="K120" s="5" t="n"/>
     </row>
     <row r="121">
       <c r="B121" s="5" t="n"/>
       <c r="C121" s="5" t="n"/>
-      <c r="I121" s="5" t="n"/>
+      <c r="K121" s="5" t="n"/>
     </row>
     <row r="122">
       <c r="B122" s="5" t="n"/>
       <c r="C122" s="5" t="n"/>
-      <c r="I122" s="5" t="n"/>
+      <c r="K122" s="5" t="n"/>
     </row>
     <row r="123">
       <c r="B123" s="5" t="n"/>
       <c r="C123" s="5" t="n"/>
-      <c r="I123" s="5" t="n"/>
+      <c r="K123" s="5" t="n"/>
     </row>
     <row r="124">
       <c r="B124" s="5" t="n"/>
       <c r="C124" s="5" t="n"/>
-      <c r="I124" s="5" t="n"/>
+      <c r="K124" s="5" t="n"/>
     </row>
     <row r="125">
       <c r="B125" s="5" t="n"/>
       <c r="C125" s="5" t="n"/>
-      <c r="I125" s="5" t="n"/>
+      <c r="K125" s="5" t="n"/>
     </row>
     <row r="126">
       <c r="B126" s="5" t="n"/>
       <c r="C126" s="5" t="n"/>
-      <c r="I126" s="5" t="n"/>
+      <c r="K126" s="5" t="n"/>
     </row>
     <row r="127">
       <c r="B127" s="5" t="n"/>
       <c r="C127" s="5" t="n"/>
-      <c r="I127" s="5" t="n"/>
+      <c r="K127" s="5" t="n"/>
     </row>
     <row r="128">
       <c r="B128" s="5" t="n"/>
       <c r="C128" s="5" t="n"/>
-      <c r="I128" s="5" t="n"/>
+      <c r="K128" s="5" t="n"/>
     </row>
     <row r="129">
       <c r="B129" s="5" t="n"/>
       <c r="C129" s="5" t="n"/>
-      <c r="I129" s="5" t="n"/>
+      <c r="K129" s="5" t="n"/>
     </row>
     <row r="130">
       <c r="B130" s="5" t="n"/>
       <c r="C130" s="5" t="n"/>
-      <c r="I130" s="5" t="n"/>
+      <c r="K130" s="5" t="n"/>
     </row>
     <row r="131">
       <c r="B131" s="5" t="n"/>
       <c r="C131" s="5" t="n"/>
-      <c r="I131" s="5" t="n"/>
+      <c r="K131" s="5" t="n"/>
     </row>
     <row r="132">
       <c r="B132" s="5" t="n"/>
       <c r="C132" s="5" t="n"/>
-      <c r="I132" s="5" t="n"/>
+      <c r="K132" s="5" t="n"/>
     </row>
     <row r="133">
       <c r="B133" s="5" t="n"/>
       <c r="C133" s="5" t="n"/>
-      <c r="I133" s="5" t="n"/>
+      <c r="K133" s="5" t="n"/>
     </row>
     <row r="134">
       <c r="B134" s="5" t="n"/>
       <c r="C134" s="5" t="n"/>
-      <c r="I134" s="5" t="n"/>
+      <c r="K134" s="5" t="n"/>
     </row>
     <row r="135">
       <c r="B135" s="5" t="n"/>
       <c r="C135" s="5" t="n"/>
-      <c r="I135" s="5" t="n"/>
+      <c r="K135" s="5" t="n"/>
     </row>
     <row r="136">
       <c r="B136" s="5" t="n"/>
       <c r="C136" s="5" t="n"/>
-      <c r="I136" s="5" t="n"/>
+      <c r="K136" s="5" t="n"/>
     </row>
     <row r="137">
       <c r="B137" s="5" t="n"/>
       <c r="C137" s="5" t="n"/>
-      <c r="I137" s="5" t="n"/>
+      <c r="K137" s="5" t="n"/>
     </row>
     <row r="138">
       <c r="B138" s="5" t="n"/>
       <c r="C138" s="5" t="n"/>
-      <c r="I138" s="5" t="n"/>
+      <c r="K138" s="5" t="n"/>
     </row>
     <row r="139">
       <c r="B139" s="5" t="n"/>
       <c r="C139" s="5" t="n"/>
-      <c r="I139" s="5" t="n"/>
+      <c r="K139" s="5" t="n"/>
     </row>
     <row r="140">
       <c r="B140" s="5" t="n"/>
       <c r="C140" s="5" t="n"/>
-      <c r="I140" s="5" t="n"/>
+      <c r="K140" s="5" t="n"/>
     </row>
     <row r="141">
       <c r="B141" s="5" t="n"/>
       <c r="C141" s="5" t="n"/>
-      <c r="I141" s="5" t="n"/>
+      <c r="K141" s="5" t="n"/>
     </row>
     <row r="142">
       <c r="B142" s="5" t="n"/>
       <c r="C142" s="5" t="n"/>
-      <c r="I142" s="5" t="n"/>
+      <c r="K142" s="5" t="n"/>
     </row>
     <row r="143">
       <c r="B143" s="5" t="n"/>
       <c r="C143" s="5" t="n"/>
-      <c r="I143" s="5" t="n"/>
+      <c r="K143" s="5" t="n"/>
     </row>
     <row r="144">
       <c r="B144" s="5" t="n"/>
       <c r="C144" s="5" t="n"/>
-      <c r="I144" s="5" t="n"/>
+      <c r="K144" s="5" t="n"/>
     </row>
     <row r="145">
       <c r="B145" s="5" t="n"/>
       <c r="C145" s="5" t="n"/>
-      <c r="I145" s="5" t="n"/>
+      <c r="K145" s="5" t="n"/>
     </row>
     <row r="146">
       <c r="B146" s="5" t="n"/>
       <c r="C146" s="5" t="n"/>
-      <c r="I146" s="5" t="n"/>
+      <c r="K146" s="5" t="n"/>
     </row>
     <row r="147">
       <c r="B147" s="5" t="n"/>
       <c r="C147" s="5" t="n"/>
-      <c r="I147" s="5" t="n"/>
+      <c r="K147" s="5" t="n"/>
     </row>
     <row r="148">
       <c r="B148" s="5" t="n"/>
       <c r="C148" s="5" t="n"/>
-      <c r="I148" s="5" t="n"/>
+      <c r="K148" s="5" t="n"/>
     </row>
     <row r="149">
       <c r="B149" s="5" t="n"/>
       <c r="C149" s="5" t="n"/>
-      <c r="I149" s="5" t="n"/>
+      <c r="K149" s="5" t="n"/>
     </row>
     <row r="150">
       <c r="B150" s="5" t="n"/>
       <c r="C150" s="5" t="n"/>
-      <c r="I150" s="5" t="n"/>
+      <c r="K150" s="5" t="n"/>
     </row>
     <row r="151">
       <c r="B151" s="5" t="n"/>
       <c r="C151" s="5" t="n"/>
-      <c r="I151" s="5" t="n"/>
+      <c r="K151" s="5" t="n"/>
     </row>
     <row r="152">
       <c r="B152" s="5" t="n"/>
       <c r="C152" s="5" t="n"/>
-      <c r="I152" s="5" t="n"/>
+      <c r="K152" s="5" t="n"/>
     </row>
     <row r="153">
       <c r="B153" s="5" t="n"/>
       <c r="C153" s="5" t="n"/>
-      <c r="I153" s="5" t="n"/>
+      <c r="K153" s="5" t="n"/>
     </row>
     <row r="154">
       <c r="B154" s="5" t="n"/>
       <c r="C154" s="5" t="n"/>
-      <c r="I154" s="5" t="n"/>
+      <c r="K154" s="5" t="n"/>
     </row>
     <row r="155">
       <c r="B155" s="5" t="n"/>
       <c r="C155" s="5" t="n"/>
-      <c r="I155" s="5" t="n"/>
+      <c r="K155" s="5" t="n"/>
     </row>
     <row r="156">
       <c r="B156" s="5" t="n"/>
       <c r="C156" s="5" t="n"/>
-      <c r="I156" s="5" t="n"/>
+      <c r="K156" s="5" t="n"/>
     </row>
     <row r="157">
       <c r="B157" s="5" t="n"/>
       <c r="C157" s="5" t="n"/>
-      <c r="I157" s="5" t="n"/>
+      <c r="K157" s="5" t="n"/>
     </row>
     <row r="158">
       <c r="B158" s="5" t="n"/>
       <c r="C158" s="5" t="n"/>
-      <c r="I158" s="5" t="n"/>
+      <c r="K158" s="5" t="n"/>
     </row>
     <row r="159">
       <c r="B159" s="5" t="n"/>
       <c r="C159" s="5" t="n"/>
-      <c r="I159" s="5" t="n"/>
+      <c r="K159" s="5" t="n"/>
     </row>
     <row r="160">
       <c r="B160" s="5" t="n"/>
       <c r="C160" s="5" t="n"/>
-      <c r="I160" s="5" t="n"/>
+      <c r="K160" s="5" t="n"/>
     </row>
     <row r="161">
       <c r="B161" s="5" t="n"/>
       <c r="C161" s="5" t="n"/>
-      <c r="I161" s="5" t="n"/>
+      <c r="K161" s="5" t="n"/>
     </row>
     <row r="162">
       <c r="B162" s="5" t="n"/>
       <c r="C162" s="5" t="n"/>
-      <c r="I162" s="5" t="n"/>
+      <c r="K162" s="5" t="n"/>
     </row>
     <row r="163">
       <c r="B163" s="5" t="n"/>
       <c r="C163" s="5" t="n"/>
-      <c r="I163" s="5" t="n"/>
+      <c r="K163" s="5" t="n"/>
     </row>
     <row r="164">
       <c r="B164" s="5" t="n"/>
       <c r="C164" s="5" t="n"/>
-      <c r="I164" s="5" t="n"/>
+      <c r="K164" s="5" t="n"/>
     </row>
     <row r="165">
       <c r="B165" s="5" t="n"/>
       <c r="C165" s="5" t="n"/>
-      <c r="I165" s="5" t="n"/>
+      <c r="K165" s="5" t="n"/>
     </row>
     <row r="166">
       <c r="B166" s="5" t="n"/>
       <c r="C166" s="5" t="n"/>
-      <c r="I166" s="5" t="n"/>
+      <c r="K166" s="5" t="n"/>
     </row>
     <row r="167">
       <c r="B167" s="5" t="n"/>
       <c r="C167" s="5" t="n"/>
-      <c r="I167" s="5" t="n"/>
+      <c r="K167" s="5" t="n"/>
     </row>
     <row r="168">
       <c r="B168" s="5" t="n"/>
       <c r="C168" s="5" t="n"/>
-      <c r="I168" s="5" t="n"/>
+      <c r="K168" s="5" t="n"/>
     </row>
     <row r="169">
       <c r="B169" s="5" t="n"/>
       <c r="C169" s="5" t="n"/>
-      <c r="I169" s="5" t="n"/>
+      <c r="K169" s="5" t="n"/>
     </row>
     <row r="170">
       <c r="B170" s="5" t="n"/>
       <c r="C170" s="5" t="n"/>
-      <c r="I170" s="5" t="n"/>
+      <c r="K170" s="5" t="n"/>
     </row>
     <row r="171">
       <c r="B171" s="5" t="n"/>
       <c r="C171" s="5" t="n"/>
-      <c r="I171" s="5" t="n"/>
+      <c r="K171" s="5" t="n"/>
     </row>
     <row r="172">
       <c r="B172" s="5" t="n"/>
       <c r="C172" s="5" t="n"/>
-      <c r="I172" s="5" t="n"/>
+      <c r="K172" s="5" t="n"/>
     </row>
     <row r="173">
       <c r="B173" s="5" t="n"/>
       <c r="C173" s="5" t="n"/>
-      <c r="I173" s="5" t="n"/>
+      <c r="K173" s="5" t="n"/>
     </row>
     <row r="174">
       <c r="B174" s="5" t="n"/>
       <c r="C174" s="5" t="n"/>
-      <c r="I174" s="5" t="n"/>
+      <c r="K174" s="5" t="n"/>
     </row>
     <row r="175">
       <c r="B175" s="5" t="n"/>
       <c r="C175" s="5" t="n"/>
-      <c r="I175" s="5" t="n"/>
+      <c r="K175" s="5" t="n"/>
     </row>
     <row r="176">
       <c r="B176" s="5" t="n"/>
       <c r="C176" s="5" t="n"/>
-      <c r="I176" s="5" t="n"/>
+      <c r="K176" s="5" t="n"/>
     </row>
     <row r="177">
       <c r="B177" s="5" t="n"/>
       <c r="C177" s="5" t="n"/>
-      <c r="I177" s="5" t="n"/>
+      <c r="K177" s="5" t="n"/>
     </row>
     <row r="178">
       <c r="B178" s="5" t="n"/>
       <c r="C178" s="5" t="n"/>
-      <c r="I178" s="5" t="n"/>
+      <c r="K178" s="5" t="n"/>
     </row>
     <row r="179">
       <c r="B179" s="5" t="n"/>
       <c r="C179" s="5" t="n"/>
-      <c r="I179" s="5" t="n"/>
+      <c r="K179" s="5" t="n"/>
     </row>
     <row r="180">
       <c r="B180" s="5" t="n"/>
       <c r="C180" s="5" t="n"/>
-      <c r="I180" s="5" t="n"/>
+      <c r="K180" s="5" t="n"/>
     </row>
     <row r="181">
       <c r="B181" s="5" t="n"/>
       <c r="C181" s="5" t="n"/>
-      <c r="I181" s="5" t="n"/>
+      <c r="K181" s="5" t="n"/>
     </row>
     <row r="182">
       <c r="B182" s="5" t="n"/>
       <c r="C182" s="5" t="n"/>
-      <c r="I182" s="5" t="n"/>
+      <c r="K182" s="5" t="n"/>
     </row>
     <row r="183">
       <c r="B183" s="5" t="n"/>
       <c r="C183" s="5" t="n"/>
-      <c r="I183" s="5" t="n"/>
+      <c r="K183" s="5" t="n"/>
     </row>
     <row r="184">
       <c r="B184" s="5" t="n"/>
       <c r="C184" s="5" t="n"/>
-      <c r="I184" s="5" t="n"/>
+      <c r="K184" s="5" t="n"/>
     </row>
     <row r="185">
       <c r="B185" s="5" t="n"/>
       <c r="C185" s="5" t="n"/>
-      <c r="I185" s="5" t="n"/>
+      <c r="K185" s="5" t="n"/>
     </row>
     <row r="186">
       <c r="B186" s="5" t="n"/>
       <c r="C186" s="5" t="n"/>
-      <c r="I186" s="5" t="n"/>
+      <c r="K186" s="5" t="n"/>
     </row>
     <row r="187">
       <c r="B187" s="5" t="n"/>
       <c r="C187" s="5" t="n"/>
-      <c r="I187" s="5" t="n"/>
+      <c r="K187" s="5" t="n"/>
     </row>
     <row r="188">
       <c r="B188" s="5" t="n"/>
       <c r="C188" s="5" t="n"/>
-      <c r="I188" s="5" t="n"/>
+      <c r="K188" s="5" t="n"/>
     </row>
     <row r="189">
       <c r="B189" s="5" t="n"/>
       <c r="C189" s="5" t="n"/>
-      <c r="I189" s="5" t="n"/>
+      <c r="K189" s="5" t="n"/>
     </row>
     <row r="190">
       <c r="B190" s="5" t="n"/>
       <c r="C190" s="5" t="n"/>
-      <c r="I190" s="5" t="n"/>
+      <c r="K190" s="5" t="n"/>
     </row>
     <row r="191">
       <c r="B191" s="5" t="n"/>
       <c r="C191" s="5" t="n"/>
-      <c r="I191" s="5" t="n"/>
+      <c r="K191" s="5" t="n"/>
     </row>
     <row r="192">
       <c r="B192" s="5" t="n"/>
       <c r="C192" s="5" t="n"/>
-      <c r="I192" s="5" t="n"/>
+      <c r="K192" s="5" t="n"/>
     </row>
     <row r="193">
       <c r="B193" s="5" t="n"/>
       <c r="C193" s="5" t="n"/>
-      <c r="I193" s="5" t="n"/>
+      <c r="K193" s="5" t="n"/>
     </row>
     <row r="194">
       <c r="B194" s="5" t="n"/>
       <c r="C194" s="5" t="n"/>
-      <c r="I194" s="5" t="n"/>
+      <c r="K194" s="5" t="n"/>
     </row>
     <row r="195">
       <c r="B195" s="5" t="n"/>
       <c r="C195" s="5" t="n"/>
-      <c r="I195" s="5" t="n"/>
+      <c r="K195" s="5" t="n"/>
     </row>
     <row r="196">
       <c r="B196" s="5" t="n"/>
       <c r="C196" s="5" t="n"/>
-      <c r="I196" s="5" t="n"/>
+      <c r="K196" s="5" t="n"/>
     </row>
     <row r="197">
       <c r="B197" s="5" t="n"/>
       <c r="C197" s="5" t="n"/>
-      <c r="I197" s="5" t="n"/>
+      <c r="K197" s="5" t="n"/>
     </row>
     <row r="198">
       <c r="B198" s="5" t="n"/>
       <c r="C198" s="5" t="n"/>
-      <c r="I198" s="5" t="n"/>
+      <c r="K198" s="5" t="n"/>
     </row>
     <row r="199">
       <c r="B199" s="5" t="n"/>
       <c r="C199" s="5" t="n"/>
-      <c r="I199" s="5" t="n"/>
+      <c r="K199" s="5" t="n"/>
     </row>
     <row r="200">
       <c r="B200" s="5" t="n"/>
       <c r="C200" s="5" t="n"/>
-      <c r="I200" s="5" t="n"/>
+      <c r="K200" s="5" t="n"/>
     </row>
     <row r="201">
       <c r="B201" s="5" t="n"/>
       <c r="C201" s="5" t="n"/>
-      <c r="I201" s="5" t="n"/>
+      <c r="K201" s="5" t="n"/>
     </row>
     <row r="202">
       <c r="B202" s="5" t="n"/>
       <c r="C202" s="5" t="n"/>
-      <c r="I202" s="5" t="n"/>
+      <c r="K202" s="5" t="n"/>
     </row>
     <row r="203">
       <c r="B203" s="5" t="n"/>
       <c r="C203" s="5" t="n"/>
-      <c r="I203" s="5" t="n"/>
+      <c r="K203" s="5" t="n"/>
     </row>
     <row r="204">
       <c r="B204" s="5" t="n"/>
       <c r="C204" s="5" t="n"/>
-      <c r="I204" s="5" t="n"/>
+      <c r="K204" s="5" t="n"/>
     </row>
     <row r="205">
       <c r="B205" s="5" t="n"/>
       <c r="C205" s="5" t="n"/>
-      <c r="I205" s="5" t="n"/>
+      <c r="K205" s="5" t="n"/>
     </row>
     <row r="206">
       <c r="B206" s="5" t="n"/>
       <c r="C206" s="5" t="n"/>
-      <c r="I206" s="5" t="n"/>
+      <c r="K206" s="5" t="n"/>
     </row>
     <row r="207">
       <c r="B207" s="5" t="n"/>
       <c r="C207" s="5" t="n"/>
-      <c r="I207" s="5" t="n"/>
+      <c r="K207" s="5" t="n"/>
     </row>
     <row r="208">
       <c r="B208" s="5" t="n"/>
       <c r="C208" s="5" t="n"/>
-      <c r="I208" s="5" t="n"/>
+      <c r="K208" s="5" t="n"/>
     </row>
     <row r="209">
       <c r="B209" s="5" t="n"/>
       <c r="C209" s="5" t="n"/>
-      <c r="I209" s="5" t="n"/>
+      <c r="K209" s="5" t="n"/>
     </row>
     <row r="210">
       <c r="B210" s="5" t="n"/>
       <c r="C210" s="5" t="n"/>
-      <c r="I210" s="5" t="n"/>
+      <c r="K210" s="5" t="n"/>
     </row>
     <row r="211">
       <c r="B211" s="5" t="n"/>
       <c r="C211" s="5" t="n"/>
-      <c r="I211" s="5" t="n"/>
+      <c r="K211" s="5" t="n"/>
     </row>
     <row r="212">
       <c r="B212" s="5" t="n"/>
       <c r="C212" s="5" t="n"/>
-      <c r="I212" s="5" t="n"/>
+      <c r="K212" s="5" t="n"/>
     </row>
     <row r="213">
       <c r="B213" s="5" t="n"/>
       <c r="C213" s="5" t="n"/>
-      <c r="I213" s="5" t="n"/>
+      <c r="K213" s="5" t="n"/>
     </row>
     <row r="214">
       <c r="B214" s="5" t="n"/>
       <c r="C214" s="5" t="n"/>
-      <c r="I214" s="5" t="n"/>
+      <c r="K214" s="5" t="n"/>
     </row>
     <row r="215">
       <c r="B215" s="5" t="n"/>
       <c r="C215" s="5" t="n"/>
-      <c r="I215" s="5" t="n"/>
+      <c r="K215" s="5" t="n"/>
     </row>
     <row r="216">
       <c r="B216" s="5" t="n"/>
       <c r="C216" s="5" t="n"/>
-      <c r="I216" s="5" t="n"/>
+      <c r="K216" s="5" t="n"/>
     </row>
     <row r="217">
       <c r="B217" s="5" t="n"/>
       <c r="C217" s="5" t="n"/>
-      <c r="I217" s="5" t="n"/>
+      <c r="K217" s="5" t="n"/>
     </row>
     <row r="218">
       <c r="B218" s="5" t="n"/>
       <c r="C218" s="5" t="n"/>
-      <c r="I218" s="5" t="n"/>
+      <c r="K218" s="5" t="n"/>
     </row>
     <row r="219">
       <c r="B219" s="5" t="n"/>
       <c r="C219" s="5" t="n"/>
-      <c r="I219" s="5" t="n"/>
+      <c r="K219" s="5" t="n"/>
     </row>
     <row r="220">
       <c r="B220" s="5" t="n"/>
       <c r="C220" s="5" t="n"/>
-      <c r="I220" s="5" t="n"/>
+      <c r="K220" s="5" t="n"/>
     </row>
     <row r="221">
       <c r="B221" s="5" t="n"/>
       <c r="C221" s="5" t="n"/>
-      <c r="I221" s="5" t="n"/>
+      <c r="K221" s="5" t="n"/>
     </row>
     <row r="222">
       <c r="B222" s="5" t="n"/>
       <c r="C222" s="5" t="n"/>
-      <c r="I222" s="5" t="n"/>
+      <c r="K222" s="5" t="n"/>
     </row>
     <row r="223">
       <c r="B223" s="5" t="n"/>
       <c r="C223" s="5" t="n"/>
-      <c r="I223" s="5" t="n"/>
+      <c r="K223" s="5" t="n"/>
     </row>
     <row r="224">
       <c r="B224" s="5" t="n"/>
       <c r="C224" s="5" t="n"/>
-      <c r="I224" s="5" t="n"/>
+      <c r="K224" s="5" t="n"/>
     </row>
     <row r="225">
       <c r="B225" s="5" t="n"/>
       <c r="C225" s="5" t="n"/>
-      <c r="I225" s="5" t="n"/>
+      <c r="K225" s="5" t="n"/>
     </row>
     <row r="226">
       <c r="B226" s="5" t="n"/>
       <c r="C226" s="5" t="n"/>
-      <c r="I226" s="5" t="n"/>
+      <c r="K226" s="5" t="n"/>
     </row>
     <row r="227">
       <c r="B227" s="5" t="n"/>
       <c r="C227" s="5" t="n"/>
-      <c r="I227" s="5" t="n"/>
+      <c r="K227" s="5" t="n"/>
     </row>
     <row r="228">
       <c r="B228" s="5" t="n"/>
       <c r="C228" s="5" t="n"/>
-      <c r="I228" s="5" t="n"/>
+      <c r="K228" s="5" t="n"/>
     </row>
     <row r="229">
       <c r="B229" s="5" t="n"/>
       <c r="C229" s="5" t="n"/>
-      <c r="I229" s="5" t="n"/>
+      <c r="K229" s="5" t="n"/>
     </row>
     <row r="230">
       <c r="B230" s="5" t="n"/>
       <c r="C230" s="5" t="n"/>
-      <c r="I230" s="5" t="n"/>
+      <c r="K230" s="5" t="n"/>
     </row>
     <row r="231">
       <c r="B231" s="5" t="n"/>
       <c r="C231" s="5" t="n"/>
-      <c r="I231" s="5" t="n"/>
+      <c r="K231" s="5" t="n"/>
     </row>
     <row r="232">
       <c r="B232" s="5" t="n"/>
       <c r="C232" s="5" t="n"/>
-      <c r="I232" s="5" t="n"/>
+      <c r="K232" s="5" t="n"/>
     </row>
     <row r="233">
       <c r="B233" s="5" t="n"/>
       <c r="C233" s="5" t="n"/>
-      <c r="I233" s="5" t="n"/>
+      <c r="K233" s="5" t="n"/>
     </row>
     <row r="234">
       <c r="B234" s="5" t="n"/>
       <c r="C234" s="5" t="n"/>
-      <c r="I234" s="5" t="n"/>
+      <c r="K234" s="5" t="n"/>
     </row>
     <row r="235">
       <c r="B235" s="5" t="n"/>
       <c r="C235" s="5" t="n"/>
-      <c r="I235" s="5" t="n"/>
+      <c r="K235" s="5" t="n"/>
     </row>
     <row r="236">
       <c r="B236" s="5" t="n"/>
       <c r="C236" s="5" t="n"/>
-      <c r="I236" s="5" t="n"/>
+      <c r="K236" s="5" t="n"/>
     </row>
     <row r="237">
       <c r="B237" s="5" t="n"/>
       <c r="C237" s="5" t="n"/>
-      <c r="I237" s="5" t="n"/>
+      <c r="K237" s="5" t="n"/>
     </row>
     <row r="238">
       <c r="B238" s="5" t="n"/>
       <c r="C238" s="5" t="n"/>
-      <c r="I238" s="5" t="n"/>
+      <c r="K238" s="5" t="n"/>
     </row>
     <row r="239">
       <c r="B239" s="5" t="n"/>
       <c r="C239" s="5" t="n"/>
-      <c r="I239" s="5" t="n"/>
+      <c r="K239" s="5" t="n"/>
     </row>
     <row r="240">
       <c r="B240" s="5" t="n"/>
       <c r="C240" s="5" t="n"/>
-      <c r="I240" s="5" t="n"/>
+      <c r="K240" s="5" t="n"/>
     </row>
     <row r="241">
       <c r="B241" s="5" t="n"/>
       <c r="C241" s="5" t="n"/>
-      <c r="I241" s="5" t="n"/>
+      <c r="K241" s="5" t="n"/>
     </row>
     <row r="242">
       <c r="B242" s="5" t="n"/>
       <c r="C242" s="5" t="n"/>
-      <c r="I242" s="5" t="n"/>
+      <c r="K242" s="5" t="n"/>
     </row>
     <row r="243">
       <c r="B243" s="5" t="n"/>
       <c r="C243" s="5" t="n"/>
-      <c r="I243" s="5" t="n"/>
+      <c r="K243" s="5" t="n"/>
     </row>
     <row r="244">
       <c r="B244" s="5" t="n"/>
       <c r="C244" s="5" t="n"/>
-      <c r="I244" s="5" t="n"/>
+      <c r="K244" s="5" t="n"/>
     </row>
     <row r="245">
       <c r="B245" s="5" t="n"/>
       <c r="C245" s="5" t="n"/>
-      <c r="I245" s="5" t="n"/>
+      <c r="K245" s="5" t="n"/>
     </row>
     <row r="246">
       <c r="B246" s="5" t="n"/>
       <c r="C246" s="5" t="n"/>
-      <c r="I246" s="5" t="n"/>
+      <c r="K246" s="5" t="n"/>
     </row>
     <row r="247">
       <c r="B247" s="5" t="n"/>
       <c r="C247" s="5" t="n"/>
-      <c r="I247" s="5" t="n"/>
+      <c r="K247" s="5" t="n"/>
     </row>
     <row r="248">
       <c r="B248" s="5" t="n"/>
       <c r="C248" s="5" t="n"/>
-      <c r="I248" s="5" t="n"/>
+      <c r="K248" s="5" t="n"/>
     </row>
     <row r="249">
       <c r="B249" s="5" t="n"/>
       <c r="C249" s="5" t="n"/>
-      <c r="I249" s="5" t="n"/>
+      <c r="K249" s="5" t="n"/>
     </row>
     <row r="250">
       <c r="B250" s="5" t="n"/>
       <c r="C250" s="5" t="n"/>
-      <c r="I250" s="5" t="n"/>
+      <c r="K250" s="5" t="n"/>
     </row>
     <row r="251">
       <c r="B251" s="5" t="n"/>
       <c r="C251" s="5" t="n"/>
-      <c r="I251" s="5" t="n"/>
+      <c r="K251" s="5" t="n"/>
     </row>
     <row r="252">
       <c r="B252" s="5" t="n"/>
       <c r="C252" s="5" t="n"/>
-      <c r="I252" s="5" t="n"/>
+      <c r="K252" s="5" t="n"/>
     </row>
     <row r="253">
       <c r="B253" s="5" t="n"/>
       <c r="C253" s="5" t="n"/>
-      <c r="I253" s="5" t="n"/>
+      <c r="K253" s="5" t="n"/>
     </row>
     <row r="254">
       <c r="B254" s="5" t="n"/>
       <c r="C254" s="5" t="n"/>
-      <c r="I254" s="5" t="n"/>
+      <c r="K254" s="5" t="n"/>
     </row>
     <row r="255">
       <c r="B255" s="5" t="n"/>
       <c r="C255" s="5" t="n"/>
-      <c r="I255" s="5" t="n"/>
+      <c r="K255" s="5" t="n"/>
     </row>
     <row r="256">
       <c r="B256" s="5" t="n"/>
       <c r="C256" s="5" t="n"/>
-      <c r="I256" s="5" t="n"/>
+      <c r="K256" s="5" t="n"/>
     </row>
     <row r="257">
       <c r="B257" s="5" t="n"/>
       <c r="C257" s="5" t="n"/>
-      <c r="I257" s="5" t="n"/>
+      <c r="K257" s="5" t="n"/>
     </row>
     <row r="258">
       <c r="B258" s="5" t="n"/>
       <c r="C258" s="5" t="n"/>
-      <c r="I258" s="5" t="n"/>
+      <c r="K258" s="5" t="n"/>
     </row>
     <row r="259">
       <c r="B259" s="5" t="n"/>
       <c r="C259" s="5" t="n"/>
-      <c r="I259" s="5" t="n"/>
+      <c r="K259" s="5" t="n"/>
     </row>
     <row r="260">
       <c r="B260" s="5" t="n"/>
       <c r="C260" s="5" t="n"/>
-      <c r="I260" s="5" t="n"/>
+      <c r="K260" s="5" t="n"/>
     </row>
     <row r="261">
       <c r="B261" s="5" t="n"/>
       <c r="C261" s="5" t="n"/>
-      <c r="I261" s="5" t="n"/>
+      <c r="K261" s="5" t="n"/>
     </row>
     <row r="262">
       <c r="B262" s="5" t="n"/>
       <c r="C262" s="5" t="n"/>
-      <c r="I262" s="5" t="n"/>
+      <c r="K262" s="5" t="n"/>
     </row>
     <row r="263">
       <c r="B263" s="5" t="n"/>
       <c r="C263" s="5" t="n"/>
-      <c r="I263" s="5" t="n"/>
+      <c r="K263" s="5" t="n"/>
     </row>
     <row r="264">
       <c r="B264" s="5" t="n"/>
       <c r="C264" s="5" t="n"/>
-      <c r="I264" s="5" t="n"/>
+      <c r="K264" s="5" t="n"/>
     </row>
     <row r="265">
       <c r="B265" s="5" t="n"/>
       <c r="C265" s="5" t="n"/>
-      <c r="I265" s="5" t="n"/>
+      <c r="K265" s="5" t="n"/>
     </row>
     <row r="266">
       <c r="B266" s="5" t="n"/>
       <c r="C266" s="5" t="n"/>
-      <c r="I266" s="5" t="n"/>
+      <c r="K266" s="5" t="n"/>
     </row>
     <row r="267">
       <c r="B267" s="5" t="n"/>
       <c r="C267" s="5" t="n"/>
-      <c r="I267" s="5" t="n"/>
+      <c r="K267" s="5" t="n"/>
     </row>
     <row r="268">
       <c r="B268" s="5" t="n"/>
       <c r="C268" s="5" t="n"/>
-      <c r="I268" s="5" t="n"/>
+      <c r="K268" s="5" t="n"/>
     </row>
     <row r="269">
       <c r="B269" s="5" t="n"/>
       <c r="C269" s="5" t="n"/>
-      <c r="I269" s="5" t="n"/>
+      <c r="K269" s="5" t="n"/>
     </row>
     <row r="270">
       <c r="B270" s="5" t="n"/>
       <c r="C270" s="5" t="n"/>
-      <c r="I270" s="5" t="n"/>
+      <c r="K270" s="5" t="n"/>
     </row>
     <row r="271">
       <c r="B271" s="5" t="n"/>
       <c r="C271" s="5" t="n"/>
-      <c r="I271" s="5" t="n"/>
+      <c r="K271" s="5" t="n"/>
     </row>
     <row r="272">
       <c r="B272" s="5" t="n"/>
       <c r="C272" s="5" t="n"/>
-      <c r="I272" s="5" t="n"/>
+      <c r="K272" s="5" t="n"/>
     </row>
     <row r="273">
       <c r="B273" s="5" t="n"/>
       <c r="C273" s="5" t="n"/>
-      <c r="I273" s="5" t="n"/>
+      <c r="K273" s="5" t="n"/>
     </row>
     <row r="274">
       <c r="B274" s="5" t="n"/>
       <c r="C274" s="5" t="n"/>
-      <c r="I274" s="5" t="n"/>
+      <c r="K274" s="5" t="n"/>
     </row>
     <row r="275">
       <c r="B275" s="5" t="n"/>
       <c r="C275" s="5" t="n"/>
-      <c r="I275" s="5" t="n"/>
+      <c r="K275" s="5" t="n"/>
     </row>
     <row r="276">
       <c r="B276" s="5" t="n"/>
       <c r="C276" s="5" t="n"/>
-      <c r="I276" s="5" t="n"/>
+      <c r="K276" s="5" t="n"/>
     </row>
     <row r="277">
       <c r="B277" s="5" t="n"/>
       <c r="C277" s="5" t="n"/>
-      <c r="I277" s="5" t="n"/>
+      <c r="K277" s="5" t="n"/>
     </row>
     <row r="278">
       <c r="B278" s="5" t="n"/>
       <c r="C278" s="5" t="n"/>
-      <c r="I278" s="5" t="n"/>
+      <c r="K278" s="5" t="n"/>
     </row>
     <row r="279">
       <c r="B279" s="5" t="n"/>
       <c r="C279" s="5" t="n"/>
-      <c r="I279" s="5" t="n"/>
+      <c r="K279" s="5" t="n"/>
     </row>
     <row r="280">
       <c r="B280" s="5" t="n"/>
       <c r="C280" s="5" t="n"/>
-      <c r="I280" s="5" t="n"/>
+      <c r="K280" s="5" t="n"/>
     </row>
     <row r="281">
       <c r="B281" s="5" t="n"/>
       <c r="C281" s="5" t="n"/>
-      <c r="I281" s="5" t="n"/>
+      <c r="K281" s="5" t="n"/>
     </row>
     <row r="282">
       <c r="B282" s="5" t="n"/>
       <c r="C282" s="5" t="n"/>
-      <c r="I282" s="5" t="n"/>
+      <c r="K282" s="5" t="n"/>
     </row>
     <row r="283">
       <c r="B283" s="5" t="n"/>
       <c r="C283" s="5" t="n"/>
-      <c r="I283" s="5" t="n"/>
+      <c r="K283" s="5" t="n"/>
     </row>
     <row r="284">
       <c r="B284" s="5" t="n"/>
       <c r="C284" s="5" t="n"/>
-      <c r="I284" s="5" t="n"/>
+      <c r="K284" s="5" t="n"/>
     </row>
     <row r="285">
       <c r="B285" s="5" t="n"/>
       <c r="C285" s="5" t="n"/>
-      <c r="I285" s="5" t="n"/>
+      <c r="K285" s="5" t="n"/>
     </row>
     <row r="286">
       <c r="B286" s="5" t="n"/>
       <c r="C286" s="5" t="n"/>
-      <c r="I286" s="5" t="n"/>
+      <c r="K286" s="5" t="n"/>
     </row>
     <row r="287">
       <c r="B287" s="5" t="n"/>
       <c r="C287" s="5" t="n"/>
-      <c r="I287" s="5" t="n"/>
+      <c r="K287" s="5" t="n"/>
     </row>
     <row r="288">
       <c r="B288" s="5" t="n"/>
       <c r="C288" s="5" t="n"/>
-      <c r="I288" s="5" t="n"/>
+      <c r="K288" s="5" t="n"/>
     </row>
     <row r="289">
       <c r="B289" s="5" t="n"/>
       <c r="C289" s="5" t="n"/>
-      <c r="I289" s="5" t="n"/>
+      <c r="K289" s="5" t="n"/>
     </row>
     <row r="290">
       <c r="B290" s="5" t="n"/>
       <c r="C290" s="5" t="n"/>
-      <c r="I290" s="5" t="n"/>
+      <c r="K290" s="5" t="n"/>
     </row>
     <row r="291">
       <c r="B291" s="5" t="n"/>
       <c r="C291" s="5" t="n"/>
-      <c r="I291" s="5" t="n"/>
+      <c r="K291" s="5" t="n"/>
     </row>
     <row r="292">
       <c r="B292" s="5" t="n"/>
       <c r="C292" s="5" t="n"/>
-      <c r="I292" s="5" t="n"/>
+      <c r="K292" s="5" t="n"/>
     </row>
     <row r="293">
       <c r="B293" s="5" t="n"/>
       <c r="C293" s="5" t="n"/>
-      <c r="I293" s="5" t="n"/>
+      <c r="K293" s="5" t="n"/>
     </row>
     <row r="294">
       <c r="B294" s="5" t="n"/>
       <c r="C294" s="5" t="n"/>
-      <c r="I294" s="5" t="n"/>
+      <c r="K294" s="5" t="n"/>
     </row>
     <row r="295">
       <c r="B295" s="5" t="n"/>
       <c r="C295" s="5" t="n"/>
-      <c r="I295" s="5" t="n"/>
+      <c r="K295" s="5" t="n"/>
     </row>
     <row r="296">
       <c r="B296" s="5" t="n"/>
       <c r="C296" s="5" t="n"/>
-      <c r="I296" s="5" t="n"/>
+      <c r="K296" s="5" t="n"/>
     </row>
     <row r="297">
       <c r="B297" s="5" t="n"/>
       <c r="C297" s="5" t="n"/>
-      <c r="I297" s="5" t="n"/>
+      <c r="K297" s="5" t="n"/>
     </row>
     <row r="298">
       <c r="B298" s="5" t="n"/>
       <c r="C298" s="5" t="n"/>
-      <c r="I298" s="5" t="n"/>
+      <c r="K298" s="5" t="n"/>
     </row>
     <row r="299">
       <c r="B299" s="5" t="n"/>
       <c r="C299" s="5" t="n"/>
-      <c r="I299" s="5" t="n"/>
+      <c r="K299" s="5" t="n"/>
     </row>
     <row r="300">
       <c r="B300" s="5" t="n"/>
       <c r="C300" s="5" t="n"/>
-      <c r="I300" s="5" t="n"/>
+      <c r="K300" s="5" t="n"/>
     </row>
     <row r="301">
       <c r="B301" s="5" t="n"/>
       <c r="C301" s="5" t="n"/>
-      <c r="I301" s="5" t="n"/>
+      <c r="K301" s="5" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="4">
@@ -2114,7 +2140,7 @@
     <dataValidation sqref="E2:E301" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="ערך לא תקין" error="יש לבחור ערך מהרשימה" type="list">
       <formula1>='רשימות'!$C$1:$C$6</formula1>
     </dataValidation>
-    <dataValidation sqref="L2:L301" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="ערך לא תקין" error="יש לבחור ערך מהרשימה" type="list">
+    <dataValidation sqref="N2:N301" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="ערך לא תקין" error="יש לבחור ערך מהרשימה" type="list">
       <formula1>='רשימות'!$D$1:$D$6</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat: vehicle columns in Tamir's order; required = plate, fuel, fueling means, driver phone
Order: plate*, fuel*, fueling means*, vehicle type, model, year, L/day, L/month,
urea/day, urea/month, driver phone*, driver name, shtifomat, dept.
Vehicle type and shtifomat become optional for the customer; since both are
required questions in the Google Form, empty is sent as "אחר" / "לא".
Same order and required set in the Excel template and import; summary table too.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/order-template.xlsx
+++ b/order-template.xlsx
@@ -478,7 +478,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>3. שטיפומט: «לא», או מספר השטיפות בחודש (1 עד 5). ריק = «לא».</t>
+          <t>3. שטיפומט: «לא», או מספר השטיפות בחודש (1 עד 5). ריק = «לא». סוג רכב ריק = «אחר».</t>
         </is>
       </c>
     </row>
@@ -560,57 +560,57 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
+          <t>מס׳ רכב *</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>סוג דלק *</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
           <t>סוג אמצעי תדלוק *</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
-        <is>
-          <t>מס׳ רכב *</t>
-        </is>
-      </c>
-      <c r="C1" s="4" t="inlineStr">
-        <is>
-          <t>מס׳ טלפון נהג</t>
-        </is>
-      </c>
-      <c r="D1" s="3" t="inlineStr">
-        <is>
-          <t>סוג דלק *</t>
-        </is>
-      </c>
-      <c r="E1" s="3" t="inlineStr">
-        <is>
-          <t>סוג הרכב *</t>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>סוג הרכב</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>דגם רכב</t>
         </is>
       </c>
       <c r="F1" s="4" t="inlineStr">
         <is>
+          <t>שנת יצור</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
           <t>הגבלה בליטרים ליום</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>הגבלה בליטרים לחודש</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>הגבלת אוריאה ליום</t>
         </is>
       </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="J1" s="4" t="inlineStr">
         <is>
           <t>הגבלת אוריאה לחודש</t>
         </is>
       </c>
-      <c r="J1" s="4" t="inlineStr">
-        <is>
-          <t>דגם רכב</t>
-        </is>
-      </c>
-      <c r="K1" s="4" t="inlineStr">
-        <is>
-          <t>שנת יצור</t>
+      <c r="K1" s="3" t="inlineStr">
+        <is>
+          <t>מס׳ טלפון נהג *</t>
         </is>
       </c>
       <c r="L1" s="4" t="inlineStr">
@@ -620,1527 +620,1527 @@
       </c>
       <c r="M1" s="4" t="inlineStr">
         <is>
+          <t>שטיפומט</t>
+        </is>
+      </c>
+      <c r="N1" s="4" t="inlineStr">
+        <is>
           <t>קוד / שם מחלקה</t>
         </is>
       </c>
-      <c r="N1" s="4" t="inlineStr">
-        <is>
-          <t>שטיפומט</t>
-        </is>
-      </c>
     </row>
     <row r="2">
-      <c r="B2" s="5" t="n"/>
-      <c r="C2" s="5" t="n"/>
+      <c r="A2" s="5" t="n"/>
+      <c r="F2" s="5" t="n"/>
       <c r="K2" s="5" t="n"/>
     </row>
     <row r="3">
-      <c r="B3" s="5" t="n"/>
-      <c r="C3" s="5" t="n"/>
+      <c r="A3" s="5" t="n"/>
+      <c r="F3" s="5" t="n"/>
       <c r="K3" s="5" t="n"/>
     </row>
     <row r="4">
-      <c r="B4" s="5" t="n"/>
-      <c r="C4" s="5" t="n"/>
+      <c r="A4" s="5" t="n"/>
+      <c r="F4" s="5" t="n"/>
       <c r="K4" s="5" t="n"/>
     </row>
     <row r="5">
-      <c r="B5" s="5" t="n"/>
-      <c r="C5" s="5" t="n"/>
+      <c r="A5" s="5" t="n"/>
+      <c r="F5" s="5" t="n"/>
       <c r="K5" s="5" t="n"/>
     </row>
     <row r="6">
-      <c r="B6" s="5" t="n"/>
-      <c r="C6" s="5" t="n"/>
+      <c r="A6" s="5" t="n"/>
+      <c r="F6" s="5" t="n"/>
       <c r="K6" s="5" t="n"/>
     </row>
     <row r="7">
-      <c r="B7" s="5" t="n"/>
-      <c r="C7" s="5" t="n"/>
+      <c r="A7" s="5" t="n"/>
+      <c r="F7" s="5" t="n"/>
       <c r="K7" s="5" t="n"/>
     </row>
     <row r="8">
-      <c r="B8" s="5" t="n"/>
-      <c r="C8" s="5" t="n"/>
+      <c r="A8" s="5" t="n"/>
+      <c r="F8" s="5" t="n"/>
       <c r="K8" s="5" t="n"/>
     </row>
     <row r="9">
-      <c r="B9" s="5" t="n"/>
-      <c r="C9" s="5" t="n"/>
+      <c r="A9" s="5" t="n"/>
+      <c r="F9" s="5" t="n"/>
       <c r="K9" s="5" t="n"/>
     </row>
     <row r="10">
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="5" t="n"/>
+      <c r="A10" s="5" t="n"/>
+      <c r="F10" s="5" t="n"/>
       <c r="K10" s="5" t="n"/>
     </row>
     <row r="11">
-      <c r="B11" s="5" t="n"/>
-      <c r="C11" s="5" t="n"/>
+      <c r="A11" s="5" t="n"/>
+      <c r="F11" s="5" t="n"/>
       <c r="K11" s="5" t="n"/>
     </row>
     <row r="12">
-      <c r="B12" s="5" t="n"/>
-      <c r="C12" s="5" t="n"/>
+      <c r="A12" s="5" t="n"/>
+      <c r="F12" s="5" t="n"/>
       <c r="K12" s="5" t="n"/>
     </row>
     <row r="13">
-      <c r="B13" s="5" t="n"/>
-      <c r="C13" s="5" t="n"/>
+      <c r="A13" s="5" t="n"/>
+      <c r="F13" s="5" t="n"/>
       <c r="K13" s="5" t="n"/>
     </row>
     <row r="14">
-      <c r="B14" s="5" t="n"/>
-      <c r="C14" s="5" t="n"/>
+      <c r="A14" s="5" t="n"/>
+      <c r="F14" s="5" t="n"/>
       <c r="K14" s="5" t="n"/>
     </row>
     <row r="15">
-      <c r="B15" s="5" t="n"/>
-      <c r="C15" s="5" t="n"/>
+      <c r="A15" s="5" t="n"/>
+      <c r="F15" s="5" t="n"/>
       <c r="K15" s="5" t="n"/>
     </row>
     <row r="16">
-      <c r="B16" s="5" t="n"/>
-      <c r="C16" s="5" t="n"/>
+      <c r="A16" s="5" t="n"/>
+      <c r="F16" s="5" t="n"/>
       <c r="K16" s="5" t="n"/>
     </row>
     <row r="17">
-      <c r="B17" s="5" t="n"/>
-      <c r="C17" s="5" t="n"/>
+      <c r="A17" s="5" t="n"/>
+      <c r="F17" s="5" t="n"/>
       <c r="K17" s="5" t="n"/>
     </row>
     <row r="18">
-      <c r="B18" s="5" t="n"/>
-      <c r="C18" s="5" t="n"/>
+      <c r="A18" s="5" t="n"/>
+      <c r="F18" s="5" t="n"/>
       <c r="K18" s="5" t="n"/>
     </row>
     <row r="19">
-      <c r="B19" s="5" t="n"/>
-      <c r="C19" s="5" t="n"/>
+      <c r="A19" s="5" t="n"/>
+      <c r="F19" s="5" t="n"/>
       <c r="K19" s="5" t="n"/>
     </row>
     <row r="20">
-      <c r="B20" s="5" t="n"/>
-      <c r="C20" s="5" t="n"/>
+      <c r="A20" s="5" t="n"/>
+      <c r="F20" s="5" t="n"/>
       <c r="K20" s="5" t="n"/>
     </row>
     <row r="21">
-      <c r="B21" s="5" t="n"/>
-      <c r="C21" s="5" t="n"/>
+      <c r="A21" s="5" t="n"/>
+      <c r="F21" s="5" t="n"/>
       <c r="K21" s="5" t="n"/>
     </row>
     <row r="22">
-      <c r="B22" s="5" t="n"/>
-      <c r="C22" s="5" t="n"/>
+      <c r="A22" s="5" t="n"/>
+      <c r="F22" s="5" t="n"/>
       <c r="K22" s="5" t="n"/>
     </row>
     <row r="23">
-      <c r="B23" s="5" t="n"/>
-      <c r="C23" s="5" t="n"/>
+      <c r="A23" s="5" t="n"/>
+      <c r="F23" s="5" t="n"/>
       <c r="K23" s="5" t="n"/>
     </row>
     <row r="24">
-      <c r="B24" s="5" t="n"/>
-      <c r="C24" s="5" t="n"/>
+      <c r="A24" s="5" t="n"/>
+      <c r="F24" s="5" t="n"/>
       <c r="K24" s="5" t="n"/>
     </row>
     <row r="25">
-      <c r="B25" s="5" t="n"/>
-      <c r="C25" s="5" t="n"/>
+      <c r="A25" s="5" t="n"/>
+      <c r="F25" s="5" t="n"/>
       <c r="K25" s="5" t="n"/>
     </row>
     <row r="26">
-      <c r="B26" s="5" t="n"/>
-      <c r="C26" s="5" t="n"/>
+      <c r="A26" s="5" t="n"/>
+      <c r="F26" s="5" t="n"/>
       <c r="K26" s="5" t="n"/>
     </row>
     <row r="27">
-      <c r="B27" s="5" t="n"/>
-      <c r="C27" s="5" t="n"/>
+      <c r="A27" s="5" t="n"/>
+      <c r="F27" s="5" t="n"/>
       <c r="K27" s="5" t="n"/>
     </row>
     <row r="28">
-      <c r="B28" s="5" t="n"/>
-      <c r="C28" s="5" t="n"/>
+      <c r="A28" s="5" t="n"/>
+      <c r="F28" s="5" t="n"/>
       <c r="K28" s="5" t="n"/>
     </row>
     <row r="29">
-      <c r="B29" s="5" t="n"/>
-      <c r="C29" s="5" t="n"/>
+      <c r="A29" s="5" t="n"/>
+      <c r="F29" s="5" t="n"/>
       <c r="K29" s="5" t="n"/>
     </row>
     <row r="30">
-      <c r="B30" s="5" t="n"/>
-      <c r="C30" s="5" t="n"/>
+      <c r="A30" s="5" t="n"/>
+      <c r="F30" s="5" t="n"/>
       <c r="K30" s="5" t="n"/>
     </row>
     <row r="31">
-      <c r="B31" s="5" t="n"/>
-      <c r="C31" s="5" t="n"/>
+      <c r="A31" s="5" t="n"/>
+      <c r="F31" s="5" t="n"/>
       <c r="K31" s="5" t="n"/>
     </row>
     <row r="32">
-      <c r="B32" s="5" t="n"/>
-      <c r="C32" s="5" t="n"/>
+      <c r="A32" s="5" t="n"/>
+      <c r="F32" s="5" t="n"/>
       <c r="K32" s="5" t="n"/>
     </row>
     <row r="33">
-      <c r="B33" s="5" t="n"/>
-      <c r="C33" s="5" t="n"/>
+      <c r="A33" s="5" t="n"/>
+      <c r="F33" s="5" t="n"/>
       <c r="K33" s="5" t="n"/>
     </row>
     <row r="34">
-      <c r="B34" s="5" t="n"/>
-      <c r="C34" s="5" t="n"/>
+      <c r="A34" s="5" t="n"/>
+      <c r="F34" s="5" t="n"/>
       <c r="K34" s="5" t="n"/>
     </row>
     <row r="35">
-      <c r="B35" s="5" t="n"/>
-      <c r="C35" s="5" t="n"/>
+      <c r="A35" s="5" t="n"/>
+      <c r="F35" s="5" t="n"/>
       <c r="K35" s="5" t="n"/>
     </row>
     <row r="36">
-      <c r="B36" s="5" t="n"/>
-      <c r="C36" s="5" t="n"/>
+      <c r="A36" s="5" t="n"/>
+      <c r="F36" s="5" t="n"/>
       <c r="K36" s="5" t="n"/>
     </row>
     <row r="37">
-      <c r="B37" s="5" t="n"/>
-      <c r="C37" s="5" t="n"/>
+      <c r="A37" s="5" t="n"/>
+      <c r="F37" s="5" t="n"/>
       <c r="K37" s="5" t="n"/>
     </row>
     <row r="38">
-      <c r="B38" s="5" t="n"/>
-      <c r="C38" s="5" t="n"/>
+      <c r="A38" s="5" t="n"/>
+      <c r="F38" s="5" t="n"/>
       <c r="K38" s="5" t="n"/>
     </row>
     <row r="39">
-      <c r="B39" s="5" t="n"/>
-      <c r="C39" s="5" t="n"/>
+      <c r="A39" s="5" t="n"/>
+      <c r="F39" s="5" t="n"/>
       <c r="K39" s="5" t="n"/>
     </row>
     <row r="40">
-      <c r="B40" s="5" t="n"/>
-      <c r="C40" s="5" t="n"/>
+      <c r="A40" s="5" t="n"/>
+      <c r="F40" s="5" t="n"/>
       <c r="K40" s="5" t="n"/>
     </row>
     <row r="41">
-      <c r="B41" s="5" t="n"/>
-      <c r="C41" s="5" t="n"/>
+      <c r="A41" s="5" t="n"/>
+      <c r="F41" s="5" t="n"/>
       <c r="K41" s="5" t="n"/>
     </row>
     <row r="42">
-      <c r="B42" s="5" t="n"/>
-      <c r="C42" s="5" t="n"/>
+      <c r="A42" s="5" t="n"/>
+      <c r="F42" s="5" t="n"/>
       <c r="K42" s="5" t="n"/>
     </row>
     <row r="43">
-      <c r="B43" s="5" t="n"/>
-      <c r="C43" s="5" t="n"/>
+      <c r="A43" s="5" t="n"/>
+      <c r="F43" s="5" t="n"/>
       <c r="K43" s="5" t="n"/>
     </row>
     <row r="44">
-      <c r="B44" s="5" t="n"/>
-      <c r="C44" s="5" t="n"/>
+      <c r="A44" s="5" t="n"/>
+      <c r="F44" s="5" t="n"/>
       <c r="K44" s="5" t="n"/>
     </row>
     <row r="45">
-      <c r="B45" s="5" t="n"/>
-      <c r="C45" s="5" t="n"/>
+      <c r="A45" s="5" t="n"/>
+      <c r="F45" s="5" t="n"/>
       <c r="K45" s="5" t="n"/>
     </row>
     <row r="46">
-      <c r="B46" s="5" t="n"/>
-      <c r="C46" s="5" t="n"/>
+      <c r="A46" s="5" t="n"/>
+      <c r="F46" s="5" t="n"/>
       <c r="K46" s="5" t="n"/>
     </row>
     <row r="47">
-      <c r="B47" s="5" t="n"/>
-      <c r="C47" s="5" t="n"/>
+      <c r="A47" s="5" t="n"/>
+      <c r="F47" s="5" t="n"/>
       <c r="K47" s="5" t="n"/>
     </row>
     <row r="48">
-      <c r="B48" s="5" t="n"/>
-      <c r="C48" s="5" t="n"/>
+      <c r="A48" s="5" t="n"/>
+      <c r="F48" s="5" t="n"/>
       <c r="K48" s="5" t="n"/>
     </row>
     <row r="49">
-      <c r="B49" s="5" t="n"/>
-      <c r="C49" s="5" t="n"/>
+      <c r="A49" s="5" t="n"/>
+      <c r="F49" s="5" t="n"/>
       <c r="K49" s="5" t="n"/>
     </row>
     <row r="50">
-      <c r="B50" s="5" t="n"/>
-      <c r="C50" s="5" t="n"/>
+      <c r="A50" s="5" t="n"/>
+      <c r="F50" s="5" t="n"/>
       <c r="K50" s="5" t="n"/>
     </row>
     <row r="51">
-      <c r="B51" s="5" t="n"/>
-      <c r="C51" s="5" t="n"/>
+      <c r="A51" s="5" t="n"/>
+      <c r="F51" s="5" t="n"/>
       <c r="K51" s="5" t="n"/>
     </row>
     <row r="52">
-      <c r="B52" s="5" t="n"/>
-      <c r="C52" s="5" t="n"/>
+      <c r="A52" s="5" t="n"/>
+      <c r="F52" s="5" t="n"/>
       <c r="K52" s="5" t="n"/>
     </row>
     <row r="53">
-      <c r="B53" s="5" t="n"/>
-      <c r="C53" s="5" t="n"/>
+      <c r="A53" s="5" t="n"/>
+      <c r="F53" s="5" t="n"/>
       <c r="K53" s="5" t="n"/>
     </row>
     <row r="54">
-      <c r="B54" s="5" t="n"/>
-      <c r="C54" s="5" t="n"/>
+      <c r="A54" s="5" t="n"/>
+      <c r="F54" s="5" t="n"/>
       <c r="K54" s="5" t="n"/>
     </row>
     <row r="55">
-      <c r="B55" s="5" t="n"/>
-      <c r="C55" s="5" t="n"/>
+      <c r="A55" s="5" t="n"/>
+      <c r="F55" s="5" t="n"/>
       <c r="K55" s="5" t="n"/>
     </row>
     <row r="56">
-      <c r="B56" s="5" t="n"/>
-      <c r="C56" s="5" t="n"/>
+      <c r="A56" s="5" t="n"/>
+      <c r="F56" s="5" t="n"/>
       <c r="K56" s="5" t="n"/>
     </row>
     <row r="57">
-      <c r="B57" s="5" t="n"/>
-      <c r="C57" s="5" t="n"/>
+      <c r="A57" s="5" t="n"/>
+      <c r="F57" s="5" t="n"/>
       <c r="K57" s="5" t="n"/>
     </row>
     <row r="58">
-      <c r="B58" s="5" t="n"/>
-      <c r="C58" s="5" t="n"/>
+      <c r="A58" s="5" t="n"/>
+      <c r="F58" s="5" t="n"/>
       <c r="K58" s="5" t="n"/>
     </row>
     <row r="59">
-      <c r="B59" s="5" t="n"/>
-      <c r="C59" s="5" t="n"/>
+      <c r="A59" s="5" t="n"/>
+      <c r="F59" s="5" t="n"/>
       <c r="K59" s="5" t="n"/>
     </row>
     <row r="60">
-      <c r="B60" s="5" t="n"/>
-      <c r="C60" s="5" t="n"/>
+      <c r="A60" s="5" t="n"/>
+      <c r="F60" s="5" t="n"/>
       <c r="K60" s="5" t="n"/>
     </row>
     <row r="61">
-      <c r="B61" s="5" t="n"/>
-      <c r="C61" s="5" t="n"/>
+      <c r="A61" s="5" t="n"/>
+      <c r="F61" s="5" t="n"/>
       <c r="K61" s="5" t="n"/>
     </row>
     <row r="62">
-      <c r="B62" s="5" t="n"/>
-      <c r="C62" s="5" t="n"/>
+      <c r="A62" s="5" t="n"/>
+      <c r="F62" s="5" t="n"/>
       <c r="K62" s="5" t="n"/>
     </row>
     <row r="63">
-      <c r="B63" s="5" t="n"/>
-      <c r="C63" s="5" t="n"/>
+      <c r="A63" s="5" t="n"/>
+      <c r="F63" s="5" t="n"/>
       <c r="K63" s="5" t="n"/>
     </row>
     <row r="64">
-      <c r="B64" s="5" t="n"/>
-      <c r="C64" s="5" t="n"/>
+      <c r="A64" s="5" t="n"/>
+      <c r="F64" s="5" t="n"/>
       <c r="K64" s="5" t="n"/>
     </row>
     <row r="65">
-      <c r="B65" s="5" t="n"/>
-      <c r="C65" s="5" t="n"/>
+      <c r="A65" s="5" t="n"/>
+      <c r="F65" s="5" t="n"/>
       <c r="K65" s="5" t="n"/>
     </row>
     <row r="66">
-      <c r="B66" s="5" t="n"/>
-      <c r="C66" s="5" t="n"/>
+      <c r="A66" s="5" t="n"/>
+      <c r="F66" s="5" t="n"/>
       <c r="K66" s="5" t="n"/>
     </row>
     <row r="67">
-      <c r="B67" s="5" t="n"/>
-      <c r="C67" s="5" t="n"/>
+      <c r="A67" s="5" t="n"/>
+      <c r="F67" s="5" t="n"/>
       <c r="K67" s="5" t="n"/>
     </row>
     <row r="68">
-      <c r="B68" s="5" t="n"/>
-      <c r="C68" s="5" t="n"/>
+      <c r="A68" s="5" t="n"/>
+      <c r="F68" s="5" t="n"/>
       <c r="K68" s="5" t="n"/>
     </row>
     <row r="69">
-      <c r="B69" s="5" t="n"/>
-      <c r="C69" s="5" t="n"/>
+      <c r="A69" s="5" t="n"/>
+      <c r="F69" s="5" t="n"/>
       <c r="K69" s="5" t="n"/>
     </row>
     <row r="70">
-      <c r="B70" s="5" t="n"/>
-      <c r="C70" s="5" t="n"/>
+      <c r="A70" s="5" t="n"/>
+      <c r="F70" s="5" t="n"/>
       <c r="K70" s="5" t="n"/>
     </row>
     <row r="71">
-      <c r="B71" s="5" t="n"/>
-      <c r="C71" s="5" t="n"/>
+      <c r="A71" s="5" t="n"/>
+      <c r="F71" s="5" t="n"/>
       <c r="K71" s="5" t="n"/>
     </row>
     <row r="72">
-      <c r="B72" s="5" t="n"/>
-      <c r="C72" s="5" t="n"/>
+      <c r="A72" s="5" t="n"/>
+      <c r="F72" s="5" t="n"/>
       <c r="K72" s="5" t="n"/>
     </row>
     <row r="73">
-      <c r="B73" s="5" t="n"/>
-      <c r="C73" s="5" t="n"/>
+      <c r="A73" s="5" t="n"/>
+      <c r="F73" s="5" t="n"/>
       <c r="K73" s="5" t="n"/>
     </row>
     <row r="74">
-      <c r="B74" s="5" t="n"/>
-      <c r="C74" s="5" t="n"/>
+      <c r="A74" s="5" t="n"/>
+      <c r="F74" s="5" t="n"/>
       <c r="K74" s="5" t="n"/>
     </row>
     <row r="75">
-      <c r="B75" s="5" t="n"/>
-      <c r="C75" s="5" t="n"/>
+      <c r="A75" s="5" t="n"/>
+      <c r="F75" s="5" t="n"/>
       <c r="K75" s="5" t="n"/>
     </row>
     <row r="76">
-      <c r="B76" s="5" t="n"/>
-      <c r="C76" s="5" t="n"/>
+      <c r="A76" s="5" t="n"/>
+      <c r="F76" s="5" t="n"/>
       <c r="K76" s="5" t="n"/>
     </row>
     <row r="77">
-      <c r="B77" s="5" t="n"/>
-      <c r="C77" s="5" t="n"/>
+      <c r="A77" s="5" t="n"/>
+      <c r="F77" s="5" t="n"/>
       <c r="K77" s="5" t="n"/>
     </row>
     <row r="78">
-      <c r="B78" s="5" t="n"/>
-      <c r="C78" s="5" t="n"/>
+      <c r="A78" s="5" t="n"/>
+      <c r="F78" s="5" t="n"/>
       <c r="K78" s="5" t="n"/>
     </row>
     <row r="79">
-      <c r="B79" s="5" t="n"/>
-      <c r="C79" s="5" t="n"/>
+      <c r="A79" s="5" t="n"/>
+      <c r="F79" s="5" t="n"/>
       <c r="K79" s="5" t="n"/>
     </row>
     <row r="80">
-      <c r="B80" s="5" t="n"/>
-      <c r="C80" s="5" t="n"/>
+      <c r="A80" s="5" t="n"/>
+      <c r="F80" s="5" t="n"/>
       <c r="K80" s="5" t="n"/>
     </row>
     <row r="81">
-      <c r="B81" s="5" t="n"/>
-      <c r="C81" s="5" t="n"/>
+      <c r="A81" s="5" t="n"/>
+      <c r="F81" s="5" t="n"/>
       <c r="K81" s="5" t="n"/>
     </row>
     <row r="82">
-      <c r="B82" s="5" t="n"/>
-      <c r="C82" s="5" t="n"/>
+      <c r="A82" s="5" t="n"/>
+      <c r="F82" s="5" t="n"/>
       <c r="K82" s="5" t="n"/>
     </row>
     <row r="83">
-      <c r="B83" s="5" t="n"/>
-      <c r="C83" s="5" t="n"/>
+      <c r="A83" s="5" t="n"/>
+      <c r="F83" s="5" t="n"/>
       <c r="K83" s="5" t="n"/>
     </row>
     <row r="84">
-      <c r="B84" s="5" t="n"/>
-      <c r="C84" s="5" t="n"/>
+      <c r="A84" s="5" t="n"/>
+      <c r="F84" s="5" t="n"/>
       <c r="K84" s="5" t="n"/>
     </row>
     <row r="85">
-      <c r="B85" s="5" t="n"/>
-      <c r="C85" s="5" t="n"/>
+      <c r="A85" s="5" t="n"/>
+      <c r="F85" s="5" t="n"/>
       <c r="K85" s="5" t="n"/>
     </row>
     <row r="86">
-      <c r="B86" s="5" t="n"/>
-      <c r="C86" s="5" t="n"/>
+      <c r="A86" s="5" t="n"/>
+      <c r="F86" s="5" t="n"/>
       <c r="K86" s="5" t="n"/>
     </row>
     <row r="87">
-      <c r="B87" s="5" t="n"/>
-      <c r="C87" s="5" t="n"/>
+      <c r="A87" s="5" t="n"/>
+      <c r="F87" s="5" t="n"/>
       <c r="K87" s="5" t="n"/>
     </row>
     <row r="88">
-      <c r="B88" s="5" t="n"/>
-      <c r="C88" s="5" t="n"/>
+      <c r="A88" s="5" t="n"/>
+      <c r="F88" s="5" t="n"/>
       <c r="K88" s="5" t="n"/>
     </row>
     <row r="89">
-      <c r="B89" s="5" t="n"/>
-      <c r="C89" s="5" t="n"/>
+      <c r="A89" s="5" t="n"/>
+      <c r="F89" s="5" t="n"/>
       <c r="K89" s="5" t="n"/>
     </row>
     <row r="90">
-      <c r="B90" s="5" t="n"/>
-      <c r="C90" s="5" t="n"/>
+      <c r="A90" s="5" t="n"/>
+      <c r="F90" s="5" t="n"/>
       <c r="K90" s="5" t="n"/>
     </row>
     <row r="91">
-      <c r="B91" s="5" t="n"/>
-      <c r="C91" s="5" t="n"/>
+      <c r="A91" s="5" t="n"/>
+      <c r="F91" s="5" t="n"/>
       <c r="K91" s="5" t="n"/>
     </row>
     <row r="92">
-      <c r="B92" s="5" t="n"/>
-      <c r="C92" s="5" t="n"/>
+      <c r="A92" s="5" t="n"/>
+      <c r="F92" s="5" t="n"/>
       <c r="K92" s="5" t="n"/>
     </row>
     <row r="93">
-      <c r="B93" s="5" t="n"/>
-      <c r="C93" s="5" t="n"/>
+      <c r="A93" s="5" t="n"/>
+      <c r="F93" s="5" t="n"/>
       <c r="K93" s="5" t="n"/>
     </row>
     <row r="94">
-      <c r="B94" s="5" t="n"/>
-      <c r="C94" s="5" t="n"/>
+      <c r="A94" s="5" t="n"/>
+      <c r="F94" s="5" t="n"/>
       <c r="K94" s="5" t="n"/>
     </row>
     <row r="95">
-      <c r="B95" s="5" t="n"/>
-      <c r="C95" s="5" t="n"/>
+      <c r="A95" s="5" t="n"/>
+      <c r="F95" s="5" t="n"/>
       <c r="K95" s="5" t="n"/>
     </row>
     <row r="96">
-      <c r="B96" s="5" t="n"/>
-      <c r="C96" s="5" t="n"/>
+      <c r="A96" s="5" t="n"/>
+      <c r="F96" s="5" t="n"/>
       <c r="K96" s="5" t="n"/>
     </row>
     <row r="97">
-      <c r="B97" s="5" t="n"/>
-      <c r="C97" s="5" t="n"/>
+      <c r="A97" s="5" t="n"/>
+      <c r="F97" s="5" t="n"/>
       <c r="K97" s="5" t="n"/>
     </row>
     <row r="98">
-      <c r="B98" s="5" t="n"/>
-      <c r="C98" s="5" t="n"/>
+      <c r="A98" s="5" t="n"/>
+      <c r="F98" s="5" t="n"/>
       <c r="K98" s="5" t="n"/>
     </row>
     <row r="99">
-      <c r="B99" s="5" t="n"/>
-      <c r="C99" s="5" t="n"/>
+      <c r="A99" s="5" t="n"/>
+      <c r="F99" s="5" t="n"/>
       <c r="K99" s="5" t="n"/>
     </row>
     <row r="100">
-      <c r="B100" s="5" t="n"/>
-      <c r="C100" s="5" t="n"/>
+      <c r="A100" s="5" t="n"/>
+      <c r="F100" s="5" t="n"/>
       <c r="K100" s="5" t="n"/>
     </row>
     <row r="101">
-      <c r="B101" s="5" t="n"/>
-      <c r="C101" s="5" t="n"/>
+      <c r="A101" s="5" t="n"/>
+      <c r="F101" s="5" t="n"/>
       <c r="K101" s="5" t="n"/>
     </row>
     <row r="102">
-      <c r="B102" s="5" t="n"/>
-      <c r="C102" s="5" t="n"/>
+      <c r="A102" s="5" t="n"/>
+      <c r="F102" s="5" t="n"/>
       <c r="K102" s="5" t="n"/>
     </row>
     <row r="103">
-      <c r="B103" s="5" t="n"/>
-      <c r="C103" s="5" t="n"/>
+      <c r="A103" s="5" t="n"/>
+      <c r="F103" s="5" t="n"/>
       <c r="K103" s="5" t="n"/>
     </row>
     <row r="104">
-      <c r="B104" s="5" t="n"/>
-      <c r="C104" s="5" t="n"/>
+      <c r="A104" s="5" t="n"/>
+      <c r="F104" s="5" t="n"/>
       <c r="K104" s="5" t="n"/>
     </row>
     <row r="105">
-      <c r="B105" s="5" t="n"/>
-      <c r="C105" s="5" t="n"/>
+      <c r="A105" s="5" t="n"/>
+      <c r="F105" s="5" t="n"/>
       <c r="K105" s="5" t="n"/>
     </row>
     <row r="106">
-      <c r="B106" s="5" t="n"/>
-      <c r="C106" s="5" t="n"/>
+      <c r="A106" s="5" t="n"/>
+      <c r="F106" s="5" t="n"/>
       <c r="K106" s="5" t="n"/>
     </row>
     <row r="107">
-      <c r="B107" s="5" t="n"/>
-      <c r="C107" s="5" t="n"/>
+      <c r="A107" s="5" t="n"/>
+      <c r="F107" s="5" t="n"/>
       <c r="K107" s="5" t="n"/>
     </row>
     <row r="108">
-      <c r="B108" s="5" t="n"/>
-      <c r="C108" s="5" t="n"/>
+      <c r="A108" s="5" t="n"/>
+      <c r="F108" s="5" t="n"/>
       <c r="K108" s="5" t="n"/>
     </row>
     <row r="109">
-      <c r="B109" s="5" t="n"/>
-      <c r="C109" s="5" t="n"/>
+      <c r="A109" s="5" t="n"/>
+      <c r="F109" s="5" t="n"/>
       <c r="K109" s="5" t="n"/>
     </row>
     <row r="110">
-      <c r="B110" s="5" t="n"/>
-      <c r="C110" s="5" t="n"/>
+      <c r="A110" s="5" t="n"/>
+      <c r="F110" s="5" t="n"/>
       <c r="K110" s="5" t="n"/>
     </row>
     <row r="111">
-      <c r="B111" s="5" t="n"/>
-      <c r="C111" s="5" t="n"/>
+      <c r="A111" s="5" t="n"/>
+      <c r="F111" s="5" t="n"/>
       <c r="K111" s="5" t="n"/>
     </row>
     <row r="112">
-      <c r="B112" s="5" t="n"/>
-      <c r="C112" s="5" t="n"/>
+      <c r="A112" s="5" t="n"/>
+      <c r="F112" s="5" t="n"/>
       <c r="K112" s="5" t="n"/>
     </row>
     <row r="113">
-      <c r="B113" s="5" t="n"/>
-      <c r="C113" s="5" t="n"/>
+      <c r="A113" s="5" t="n"/>
+      <c r="F113" s="5" t="n"/>
       <c r="K113" s="5" t="n"/>
     </row>
     <row r="114">
-      <c r="B114" s="5" t="n"/>
-      <c r="C114" s="5" t="n"/>
+      <c r="A114" s="5" t="n"/>
+      <c r="F114" s="5" t="n"/>
       <c r="K114" s="5" t="n"/>
     </row>
     <row r="115">
-      <c r="B115" s="5" t="n"/>
-      <c r="C115" s="5" t="n"/>
+      <c r="A115" s="5" t="n"/>
+      <c r="F115" s="5" t="n"/>
       <c r="K115" s="5" t="n"/>
     </row>
     <row r="116">
-      <c r="B116" s="5" t="n"/>
-      <c r="C116" s="5" t="n"/>
+      <c r="A116" s="5" t="n"/>
+      <c r="F116" s="5" t="n"/>
       <c r="K116" s="5" t="n"/>
     </row>
     <row r="117">
-      <c r="B117" s="5" t="n"/>
-      <c r="C117" s="5" t="n"/>
+      <c r="A117" s="5" t="n"/>
+      <c r="F117" s="5" t="n"/>
       <c r="K117" s="5" t="n"/>
     </row>
     <row r="118">
-      <c r="B118" s="5" t="n"/>
-      <c r="C118" s="5" t="n"/>
+      <c r="A118" s="5" t="n"/>
+      <c r="F118" s="5" t="n"/>
       <c r="K118" s="5" t="n"/>
     </row>
     <row r="119">
-      <c r="B119" s="5" t="n"/>
-      <c r="C119" s="5" t="n"/>
+      <c r="A119" s="5" t="n"/>
+      <c r="F119" s="5" t="n"/>
       <c r="K119" s="5" t="n"/>
     </row>
     <row r="120">
-      <c r="B120" s="5" t="n"/>
-      <c r="C120" s="5" t="n"/>
+      <c r="A120" s="5" t="n"/>
+      <c r="F120" s="5" t="n"/>
       <c r="K120" s="5" t="n"/>
     </row>
     <row r="121">
-      <c r="B121" s="5" t="n"/>
-      <c r="C121" s="5" t="n"/>
+      <c r="A121" s="5" t="n"/>
+      <c r="F121" s="5" t="n"/>
       <c r="K121" s="5" t="n"/>
     </row>
     <row r="122">
-      <c r="B122" s="5" t="n"/>
-      <c r="C122" s="5" t="n"/>
+      <c r="A122" s="5" t="n"/>
+      <c r="F122" s="5" t="n"/>
       <c r="K122" s="5" t="n"/>
     </row>
     <row r="123">
-      <c r="B123" s="5" t="n"/>
-      <c r="C123" s="5" t="n"/>
+      <c r="A123" s="5" t="n"/>
+      <c r="F123" s="5" t="n"/>
       <c r="K123" s="5" t="n"/>
     </row>
     <row r="124">
-      <c r="B124" s="5" t="n"/>
-      <c r="C124" s="5" t="n"/>
+      <c r="A124" s="5" t="n"/>
+      <c r="F124" s="5" t="n"/>
       <c r="K124" s="5" t="n"/>
     </row>
     <row r="125">
-      <c r="B125" s="5" t="n"/>
-      <c r="C125" s="5" t="n"/>
+      <c r="A125" s="5" t="n"/>
+      <c r="F125" s="5" t="n"/>
       <c r="K125" s="5" t="n"/>
     </row>
     <row r="126">
-      <c r="B126" s="5" t="n"/>
-      <c r="C126" s="5" t="n"/>
+      <c r="A126" s="5" t="n"/>
+      <c r="F126" s="5" t="n"/>
       <c r="K126" s="5" t="n"/>
     </row>
     <row r="127">
-      <c r="B127" s="5" t="n"/>
-      <c r="C127" s="5" t="n"/>
+      <c r="A127" s="5" t="n"/>
+      <c r="F127" s="5" t="n"/>
       <c r="K127" s="5" t="n"/>
     </row>
     <row r="128">
-      <c r="B128" s="5" t="n"/>
-      <c r="C128" s="5" t="n"/>
+      <c r="A128" s="5" t="n"/>
+      <c r="F128" s="5" t="n"/>
       <c r="K128" s="5" t="n"/>
     </row>
     <row r="129">
-      <c r="B129" s="5" t="n"/>
-      <c r="C129" s="5" t="n"/>
+      <c r="A129" s="5" t="n"/>
+      <c r="F129" s="5" t="n"/>
       <c r="K129" s="5" t="n"/>
     </row>
     <row r="130">
-      <c r="B130" s="5" t="n"/>
-      <c r="C130" s="5" t="n"/>
+      <c r="A130" s="5" t="n"/>
+      <c r="F130" s="5" t="n"/>
       <c r="K130" s="5" t="n"/>
     </row>
     <row r="131">
-      <c r="B131" s="5" t="n"/>
-      <c r="C131" s="5" t="n"/>
+      <c r="A131" s="5" t="n"/>
+      <c r="F131" s="5" t="n"/>
       <c r="K131" s="5" t="n"/>
     </row>
     <row r="132">
-      <c r="B132" s="5" t="n"/>
-      <c r="C132" s="5" t="n"/>
+      <c r="A132" s="5" t="n"/>
+      <c r="F132" s="5" t="n"/>
       <c r="K132" s="5" t="n"/>
     </row>
     <row r="133">
-      <c r="B133" s="5" t="n"/>
-      <c r="C133" s="5" t="n"/>
+      <c r="A133" s="5" t="n"/>
+      <c r="F133" s="5" t="n"/>
       <c r="K133" s="5" t="n"/>
     </row>
     <row r="134">
-      <c r="B134" s="5" t="n"/>
-      <c r="C134" s="5" t="n"/>
+      <c r="A134" s="5" t="n"/>
+      <c r="F134" s="5" t="n"/>
       <c r="K134" s="5" t="n"/>
     </row>
     <row r="135">
-      <c r="B135" s="5" t="n"/>
-      <c r="C135" s="5" t="n"/>
+      <c r="A135" s="5" t="n"/>
+      <c r="F135" s="5" t="n"/>
       <c r="K135" s="5" t="n"/>
     </row>
     <row r="136">
-      <c r="B136" s="5" t="n"/>
-      <c r="C136" s="5" t="n"/>
+      <c r="A136" s="5" t="n"/>
+      <c r="F136" s="5" t="n"/>
       <c r="K136" s="5" t="n"/>
     </row>
     <row r="137">
-      <c r="B137" s="5" t="n"/>
-      <c r="C137" s="5" t="n"/>
+      <c r="A137" s="5" t="n"/>
+      <c r="F137" s="5" t="n"/>
       <c r="K137" s="5" t="n"/>
     </row>
     <row r="138">
-      <c r="B138" s="5" t="n"/>
-      <c r="C138" s="5" t="n"/>
+      <c r="A138" s="5" t="n"/>
+      <c r="F138" s="5" t="n"/>
       <c r="K138" s="5" t="n"/>
     </row>
     <row r="139">
-      <c r="B139" s="5" t="n"/>
-      <c r="C139" s="5" t="n"/>
+      <c r="A139" s="5" t="n"/>
+      <c r="F139" s="5" t="n"/>
       <c r="K139" s="5" t="n"/>
     </row>
     <row r="140">
-      <c r="B140" s="5" t="n"/>
-      <c r="C140" s="5" t="n"/>
+      <c r="A140" s="5" t="n"/>
+      <c r="F140" s="5" t="n"/>
       <c r="K140" s="5" t="n"/>
     </row>
     <row r="141">
-      <c r="B141" s="5" t="n"/>
-      <c r="C141" s="5" t="n"/>
+      <c r="A141" s="5" t="n"/>
+      <c r="F141" s="5" t="n"/>
       <c r="K141" s="5" t="n"/>
     </row>
     <row r="142">
-      <c r="B142" s="5" t="n"/>
-      <c r="C142" s="5" t="n"/>
+      <c r="A142" s="5" t="n"/>
+      <c r="F142" s="5" t="n"/>
       <c r="K142" s="5" t="n"/>
     </row>
     <row r="143">
-      <c r="B143" s="5" t="n"/>
-      <c r="C143" s="5" t="n"/>
+      <c r="A143" s="5" t="n"/>
+      <c r="F143" s="5" t="n"/>
       <c r="K143" s="5" t="n"/>
     </row>
     <row r="144">
-      <c r="B144" s="5" t="n"/>
-      <c r="C144" s="5" t="n"/>
+      <c r="A144" s="5" t="n"/>
+      <c r="F144" s="5" t="n"/>
       <c r="K144" s="5" t="n"/>
     </row>
     <row r="145">
-      <c r="B145" s="5" t="n"/>
-      <c r="C145" s="5" t="n"/>
+      <c r="A145" s="5" t="n"/>
+      <c r="F145" s="5" t="n"/>
       <c r="K145" s="5" t="n"/>
     </row>
     <row r="146">
-      <c r="B146" s="5" t="n"/>
-      <c r="C146" s="5" t="n"/>
+      <c r="A146" s="5" t="n"/>
+      <c r="F146" s="5" t="n"/>
       <c r="K146" s="5" t="n"/>
     </row>
     <row r="147">
-      <c r="B147" s="5" t="n"/>
-      <c r="C147" s="5" t="n"/>
+      <c r="A147" s="5" t="n"/>
+      <c r="F147" s="5" t="n"/>
       <c r="K147" s="5" t="n"/>
     </row>
     <row r="148">
-      <c r="B148" s="5" t="n"/>
-      <c r="C148" s="5" t="n"/>
+      <c r="A148" s="5" t="n"/>
+      <c r="F148" s="5" t="n"/>
       <c r="K148" s="5" t="n"/>
     </row>
     <row r="149">
-      <c r="B149" s="5" t="n"/>
-      <c r="C149" s="5" t="n"/>
+      <c r="A149" s="5" t="n"/>
+      <c r="F149" s="5" t="n"/>
       <c r="K149" s="5" t="n"/>
     </row>
     <row r="150">
-      <c r="B150" s="5" t="n"/>
-      <c r="C150" s="5" t="n"/>
+      <c r="A150" s="5" t="n"/>
+      <c r="F150" s="5" t="n"/>
       <c r="K150" s="5" t="n"/>
     </row>
     <row r="151">
-      <c r="B151" s="5" t="n"/>
-      <c r="C151" s="5" t="n"/>
+      <c r="A151" s="5" t="n"/>
+      <c r="F151" s="5" t="n"/>
       <c r="K151" s="5" t="n"/>
     </row>
     <row r="152">
-      <c r="B152" s="5" t="n"/>
-      <c r="C152" s="5" t="n"/>
+      <c r="A152" s="5" t="n"/>
+      <c r="F152" s="5" t="n"/>
       <c r="K152" s="5" t="n"/>
     </row>
     <row r="153">
-      <c r="B153" s="5" t="n"/>
-      <c r="C153" s="5" t="n"/>
+      <c r="A153" s="5" t="n"/>
+      <c r="F153" s="5" t="n"/>
       <c r="K153" s="5" t="n"/>
     </row>
     <row r="154">
-      <c r="B154" s="5" t="n"/>
-      <c r="C154" s="5" t="n"/>
+      <c r="A154" s="5" t="n"/>
+      <c r="F154" s="5" t="n"/>
       <c r="K154" s="5" t="n"/>
     </row>
     <row r="155">
-      <c r="B155" s="5" t="n"/>
-      <c r="C155" s="5" t="n"/>
+      <c r="A155" s="5" t="n"/>
+      <c r="F155" s="5" t="n"/>
       <c r="K155" s="5" t="n"/>
     </row>
     <row r="156">
-      <c r="B156" s="5" t="n"/>
-      <c r="C156" s="5" t="n"/>
+      <c r="A156" s="5" t="n"/>
+      <c r="F156" s="5" t="n"/>
       <c r="K156" s="5" t="n"/>
     </row>
     <row r="157">
-      <c r="B157" s="5" t="n"/>
-      <c r="C157" s="5" t="n"/>
+      <c r="A157" s="5" t="n"/>
+      <c r="F157" s="5" t="n"/>
       <c r="K157" s="5" t="n"/>
     </row>
     <row r="158">
-      <c r="B158" s="5" t="n"/>
-      <c r="C158" s="5" t="n"/>
+      <c r="A158" s="5" t="n"/>
+      <c r="F158" s="5" t="n"/>
       <c r="K158" s="5" t="n"/>
     </row>
     <row r="159">
-      <c r="B159" s="5" t="n"/>
-      <c r="C159" s="5" t="n"/>
+      <c r="A159" s="5" t="n"/>
+      <c r="F159" s="5" t="n"/>
       <c r="K159" s="5" t="n"/>
     </row>
     <row r="160">
-      <c r="B160" s="5" t="n"/>
-      <c r="C160" s="5" t="n"/>
+      <c r="A160" s="5" t="n"/>
+      <c r="F160" s="5" t="n"/>
       <c r="K160" s="5" t="n"/>
     </row>
     <row r="161">
-      <c r="B161" s="5" t="n"/>
-      <c r="C161" s="5" t="n"/>
+      <c r="A161" s="5" t="n"/>
+      <c r="F161" s="5" t="n"/>
       <c r="K161" s="5" t="n"/>
     </row>
     <row r="162">
-      <c r="B162" s="5" t="n"/>
-      <c r="C162" s="5" t="n"/>
+      <c r="A162" s="5" t="n"/>
+      <c r="F162" s="5" t="n"/>
       <c r="K162" s="5" t="n"/>
     </row>
     <row r="163">
-      <c r="B163" s="5" t="n"/>
-      <c r="C163" s="5" t="n"/>
+      <c r="A163" s="5" t="n"/>
+      <c r="F163" s="5" t="n"/>
       <c r="K163" s="5" t="n"/>
     </row>
     <row r="164">
-      <c r="B164" s="5" t="n"/>
-      <c r="C164" s="5" t="n"/>
+      <c r="A164" s="5" t="n"/>
+      <c r="F164" s="5" t="n"/>
       <c r="K164" s="5" t="n"/>
     </row>
     <row r="165">
-      <c r="B165" s="5" t="n"/>
-      <c r="C165" s="5" t="n"/>
+      <c r="A165" s="5" t="n"/>
+      <c r="F165" s="5" t="n"/>
       <c r="K165" s="5" t="n"/>
     </row>
     <row r="166">
-      <c r="B166" s="5" t="n"/>
-      <c r="C166" s="5" t="n"/>
+      <c r="A166" s="5" t="n"/>
+      <c r="F166" s="5" t="n"/>
       <c r="K166" s="5" t="n"/>
     </row>
     <row r="167">
-      <c r="B167" s="5" t="n"/>
-      <c r="C167" s="5" t="n"/>
+      <c r="A167" s="5" t="n"/>
+      <c r="F167" s="5" t="n"/>
       <c r="K167" s="5" t="n"/>
     </row>
     <row r="168">
-      <c r="B168" s="5" t="n"/>
-      <c r="C168" s="5" t="n"/>
+      <c r="A168" s="5" t="n"/>
+      <c r="F168" s="5" t="n"/>
       <c r="K168" s="5" t="n"/>
     </row>
     <row r="169">
-      <c r="B169" s="5" t="n"/>
-      <c r="C169" s="5" t="n"/>
+      <c r="A169" s="5" t="n"/>
+      <c r="F169" s="5" t="n"/>
       <c r="K169" s="5" t="n"/>
     </row>
     <row r="170">
-      <c r="B170" s="5" t="n"/>
-      <c r="C170" s="5" t="n"/>
+      <c r="A170" s="5" t="n"/>
+      <c r="F170" s="5" t="n"/>
       <c r="K170" s="5" t="n"/>
     </row>
     <row r="171">
-      <c r="B171" s="5" t="n"/>
-      <c r="C171" s="5" t="n"/>
+      <c r="A171" s="5" t="n"/>
+      <c r="F171" s="5" t="n"/>
       <c r="K171" s="5" t="n"/>
     </row>
     <row r="172">
-      <c r="B172" s="5" t="n"/>
-      <c r="C172" s="5" t="n"/>
+      <c r="A172" s="5" t="n"/>
+      <c r="F172" s="5" t="n"/>
       <c r="K172" s="5" t="n"/>
     </row>
     <row r="173">
-      <c r="B173" s="5" t="n"/>
-      <c r="C173" s="5" t="n"/>
+      <c r="A173" s="5" t="n"/>
+      <c r="F173" s="5" t="n"/>
       <c r="K173" s="5" t="n"/>
     </row>
     <row r="174">
-      <c r="B174" s="5" t="n"/>
-      <c r="C174" s="5" t="n"/>
+      <c r="A174" s="5" t="n"/>
+      <c r="F174" s="5" t="n"/>
       <c r="K174" s="5" t="n"/>
     </row>
     <row r="175">
-      <c r="B175" s="5" t="n"/>
-      <c r="C175" s="5" t="n"/>
+      <c r="A175" s="5" t="n"/>
+      <c r="F175" s="5" t="n"/>
       <c r="K175" s="5" t="n"/>
     </row>
     <row r="176">
-      <c r="B176" s="5" t="n"/>
-      <c r="C176" s="5" t="n"/>
+      <c r="A176" s="5" t="n"/>
+      <c r="F176" s="5" t="n"/>
       <c r="K176" s="5" t="n"/>
     </row>
     <row r="177">
-      <c r="B177" s="5" t="n"/>
-      <c r="C177" s="5" t="n"/>
+      <c r="A177" s="5" t="n"/>
+      <c r="F177" s="5" t="n"/>
       <c r="K177" s="5" t="n"/>
     </row>
     <row r="178">
-      <c r="B178" s="5" t="n"/>
-      <c r="C178" s="5" t="n"/>
+      <c r="A178" s="5" t="n"/>
+      <c r="F178" s="5" t="n"/>
       <c r="K178" s="5" t="n"/>
     </row>
     <row r="179">
-      <c r="B179" s="5" t="n"/>
-      <c r="C179" s="5" t="n"/>
+      <c r="A179" s="5" t="n"/>
+      <c r="F179" s="5" t="n"/>
       <c r="K179" s="5" t="n"/>
     </row>
     <row r="180">
-      <c r="B180" s="5" t="n"/>
-      <c r="C180" s="5" t="n"/>
+      <c r="A180" s="5" t="n"/>
+      <c r="F180" s="5" t="n"/>
       <c r="K180" s="5" t="n"/>
     </row>
     <row r="181">
-      <c r="B181" s="5" t="n"/>
-      <c r="C181" s="5" t="n"/>
+      <c r="A181" s="5" t="n"/>
+      <c r="F181" s="5" t="n"/>
       <c r="K181" s="5" t="n"/>
     </row>
     <row r="182">
-      <c r="B182" s="5" t="n"/>
-      <c r="C182" s="5" t="n"/>
+      <c r="A182" s="5" t="n"/>
+      <c r="F182" s="5" t="n"/>
       <c r="K182" s="5" t="n"/>
     </row>
     <row r="183">
-      <c r="B183" s="5" t="n"/>
-      <c r="C183" s="5" t="n"/>
+      <c r="A183" s="5" t="n"/>
+      <c r="F183" s="5" t="n"/>
       <c r="K183" s="5" t="n"/>
     </row>
     <row r="184">
-      <c r="B184" s="5" t="n"/>
-      <c r="C184" s="5" t="n"/>
+      <c r="A184" s="5" t="n"/>
+      <c r="F184" s="5" t="n"/>
       <c r="K184" s="5" t="n"/>
     </row>
     <row r="185">
-      <c r="B185" s="5" t="n"/>
-      <c r="C185" s="5" t="n"/>
+      <c r="A185" s="5" t="n"/>
+      <c r="F185" s="5" t="n"/>
       <c r="K185" s="5" t="n"/>
     </row>
     <row r="186">
-      <c r="B186" s="5" t="n"/>
-      <c r="C186" s="5" t="n"/>
+      <c r="A186" s="5" t="n"/>
+      <c r="F186" s="5" t="n"/>
       <c r="K186" s="5" t="n"/>
     </row>
     <row r="187">
-      <c r="B187" s="5" t="n"/>
-      <c r="C187" s="5" t="n"/>
+      <c r="A187" s="5" t="n"/>
+      <c r="F187" s="5" t="n"/>
       <c r="K187" s="5" t="n"/>
     </row>
     <row r="188">
-      <c r="B188" s="5" t="n"/>
-      <c r="C188" s="5" t="n"/>
+      <c r="A188" s="5" t="n"/>
+      <c r="F188" s="5" t="n"/>
       <c r="K188" s="5" t="n"/>
     </row>
     <row r="189">
-      <c r="B189" s="5" t="n"/>
-      <c r="C189" s="5" t="n"/>
+      <c r="A189" s="5" t="n"/>
+      <c r="F189" s="5" t="n"/>
       <c r="K189" s="5" t="n"/>
     </row>
     <row r="190">
-      <c r="B190" s="5" t="n"/>
-      <c r="C190" s="5" t="n"/>
+      <c r="A190" s="5" t="n"/>
+      <c r="F190" s="5" t="n"/>
       <c r="K190" s="5" t="n"/>
     </row>
     <row r="191">
-      <c r="B191" s="5" t="n"/>
-      <c r="C191" s="5" t="n"/>
+      <c r="A191" s="5" t="n"/>
+      <c r="F191" s="5" t="n"/>
       <c r="K191" s="5" t="n"/>
     </row>
     <row r="192">
-      <c r="B192" s="5" t="n"/>
-      <c r="C192" s="5" t="n"/>
+      <c r="A192" s="5" t="n"/>
+      <c r="F192" s="5" t="n"/>
       <c r="K192" s="5" t="n"/>
     </row>
     <row r="193">
-      <c r="B193" s="5" t="n"/>
-      <c r="C193" s="5" t="n"/>
+      <c r="A193" s="5" t="n"/>
+      <c r="F193" s="5" t="n"/>
       <c r="K193" s="5" t="n"/>
     </row>
     <row r="194">
-      <c r="B194" s="5" t="n"/>
-      <c r="C194" s="5" t="n"/>
+      <c r="A194" s="5" t="n"/>
+      <c r="F194" s="5" t="n"/>
       <c r="K194" s="5" t="n"/>
     </row>
     <row r="195">
-      <c r="B195" s="5" t="n"/>
-      <c r="C195" s="5" t="n"/>
+      <c r="A195" s="5" t="n"/>
+      <c r="F195" s="5" t="n"/>
       <c r="K195" s="5" t="n"/>
     </row>
     <row r="196">
-      <c r="B196" s="5" t="n"/>
-      <c r="C196" s="5" t="n"/>
+      <c r="A196" s="5" t="n"/>
+      <c r="F196" s="5" t="n"/>
       <c r="K196" s="5" t="n"/>
     </row>
     <row r="197">
-      <c r="B197" s="5" t="n"/>
-      <c r="C197" s="5" t="n"/>
+      <c r="A197" s="5" t="n"/>
+      <c r="F197" s="5" t="n"/>
       <c r="K197" s="5" t="n"/>
     </row>
     <row r="198">
-      <c r="B198" s="5" t="n"/>
-      <c r="C198" s="5" t="n"/>
+      <c r="A198" s="5" t="n"/>
+      <c r="F198" s="5" t="n"/>
       <c r="K198" s="5" t="n"/>
     </row>
     <row r="199">
-      <c r="B199" s="5" t="n"/>
-      <c r="C199" s="5" t="n"/>
+      <c r="A199" s="5" t="n"/>
+      <c r="F199" s="5" t="n"/>
       <c r="K199" s="5" t="n"/>
     </row>
     <row r="200">
-      <c r="B200" s="5" t="n"/>
-      <c r="C200" s="5" t="n"/>
+      <c r="A200" s="5" t="n"/>
+      <c r="F200" s="5" t="n"/>
       <c r="K200" s="5" t="n"/>
     </row>
     <row r="201">
-      <c r="B201" s="5" t="n"/>
-      <c r="C201" s="5" t="n"/>
+      <c r="A201" s="5" t="n"/>
+      <c r="F201" s="5" t="n"/>
       <c r="K201" s="5" t="n"/>
     </row>
     <row r="202">
-      <c r="B202" s="5" t="n"/>
-      <c r="C202" s="5" t="n"/>
+      <c r="A202" s="5" t="n"/>
+      <c r="F202" s="5" t="n"/>
       <c r="K202" s="5" t="n"/>
     </row>
     <row r="203">
-      <c r="B203" s="5" t="n"/>
-      <c r="C203" s="5" t="n"/>
+      <c r="A203" s="5" t="n"/>
+      <c r="F203" s="5" t="n"/>
       <c r="K203" s="5" t="n"/>
     </row>
     <row r="204">
-      <c r="B204" s="5" t="n"/>
-      <c r="C204" s="5" t="n"/>
+      <c r="A204" s="5" t="n"/>
+      <c r="F204" s="5" t="n"/>
       <c r="K204" s="5" t="n"/>
     </row>
     <row r="205">
-      <c r="B205" s="5" t="n"/>
-      <c r="C205" s="5" t="n"/>
+      <c r="A205" s="5" t="n"/>
+      <c r="F205" s="5" t="n"/>
       <c r="K205" s="5" t="n"/>
     </row>
     <row r="206">
-      <c r="B206" s="5" t="n"/>
-      <c r="C206" s="5" t="n"/>
+      <c r="A206" s="5" t="n"/>
+      <c r="F206" s="5" t="n"/>
       <c r="K206" s="5" t="n"/>
     </row>
     <row r="207">
-      <c r="B207" s="5" t="n"/>
-      <c r="C207" s="5" t="n"/>
+      <c r="A207" s="5" t="n"/>
+      <c r="F207" s="5" t="n"/>
       <c r="K207" s="5" t="n"/>
     </row>
     <row r="208">
-      <c r="B208" s="5" t="n"/>
-      <c r="C208" s="5" t="n"/>
+      <c r="A208" s="5" t="n"/>
+      <c r="F208" s="5" t="n"/>
       <c r="K208" s="5" t="n"/>
     </row>
     <row r="209">
-      <c r="B209" s="5" t="n"/>
-      <c r="C209" s="5" t="n"/>
+      <c r="A209" s="5" t="n"/>
+      <c r="F209" s="5" t="n"/>
       <c r="K209" s="5" t="n"/>
     </row>
     <row r="210">
-      <c r="B210" s="5" t="n"/>
-      <c r="C210" s="5" t="n"/>
+      <c r="A210" s="5" t="n"/>
+      <c r="F210" s="5" t="n"/>
       <c r="K210" s="5" t="n"/>
     </row>
     <row r="211">
-      <c r="B211" s="5" t="n"/>
-      <c r="C211" s="5" t="n"/>
+      <c r="A211" s="5" t="n"/>
+      <c r="F211" s="5" t="n"/>
       <c r="K211" s="5" t="n"/>
     </row>
     <row r="212">
-      <c r="B212" s="5" t="n"/>
-      <c r="C212" s="5" t="n"/>
+      <c r="A212" s="5" t="n"/>
+      <c r="F212" s="5" t="n"/>
       <c r="K212" s="5" t="n"/>
     </row>
     <row r="213">
-      <c r="B213" s="5" t="n"/>
-      <c r="C213" s="5" t="n"/>
+      <c r="A213" s="5" t="n"/>
+      <c r="F213" s="5" t="n"/>
       <c r="K213" s="5" t="n"/>
     </row>
     <row r="214">
-      <c r="B214" s="5" t="n"/>
-      <c r="C214" s="5" t="n"/>
+      <c r="A214" s="5" t="n"/>
+      <c r="F214" s="5" t="n"/>
       <c r="K214" s="5" t="n"/>
     </row>
     <row r="215">
-      <c r="B215" s="5" t="n"/>
-      <c r="C215" s="5" t="n"/>
+      <c r="A215" s="5" t="n"/>
+      <c r="F215" s="5" t="n"/>
       <c r="K215" s="5" t="n"/>
     </row>
     <row r="216">
-      <c r="B216" s="5" t="n"/>
-      <c r="C216" s="5" t="n"/>
+      <c r="A216" s="5" t="n"/>
+      <c r="F216" s="5" t="n"/>
       <c r="K216" s="5" t="n"/>
     </row>
     <row r="217">
-      <c r="B217" s="5" t="n"/>
-      <c r="C217" s="5" t="n"/>
+      <c r="A217" s="5" t="n"/>
+      <c r="F217" s="5" t="n"/>
       <c r="K217" s="5" t="n"/>
     </row>
     <row r="218">
-      <c r="B218" s="5" t="n"/>
-      <c r="C218" s="5" t="n"/>
+      <c r="A218" s="5" t="n"/>
+      <c r="F218" s="5" t="n"/>
       <c r="K218" s="5" t="n"/>
     </row>
     <row r="219">
-      <c r="B219" s="5" t="n"/>
-      <c r="C219" s="5" t="n"/>
+      <c r="A219" s="5" t="n"/>
+      <c r="F219" s="5" t="n"/>
       <c r="K219" s="5" t="n"/>
     </row>
     <row r="220">
-      <c r="B220" s="5" t="n"/>
-      <c r="C220" s="5" t="n"/>
+      <c r="A220" s="5" t="n"/>
+      <c r="F220" s="5" t="n"/>
       <c r="K220" s="5" t="n"/>
     </row>
     <row r="221">
-      <c r="B221" s="5" t="n"/>
-      <c r="C221" s="5" t="n"/>
+      <c r="A221" s="5" t="n"/>
+      <c r="F221" s="5" t="n"/>
       <c r="K221" s="5" t="n"/>
     </row>
     <row r="222">
-      <c r="B222" s="5" t="n"/>
-      <c r="C222" s="5" t="n"/>
+      <c r="A222" s="5" t="n"/>
+      <c r="F222" s="5" t="n"/>
       <c r="K222" s="5" t="n"/>
     </row>
     <row r="223">
-      <c r="B223" s="5" t="n"/>
-      <c r="C223" s="5" t="n"/>
+      <c r="A223" s="5" t="n"/>
+      <c r="F223" s="5" t="n"/>
       <c r="K223" s="5" t="n"/>
     </row>
     <row r="224">
-      <c r="B224" s="5" t="n"/>
-      <c r="C224" s="5" t="n"/>
+      <c r="A224" s="5" t="n"/>
+      <c r="F224" s="5" t="n"/>
       <c r="K224" s="5" t="n"/>
     </row>
     <row r="225">
-      <c r="B225" s="5" t="n"/>
-      <c r="C225" s="5" t="n"/>
+      <c r="A225" s="5" t="n"/>
+      <c r="F225" s="5" t="n"/>
       <c r="K225" s="5" t="n"/>
     </row>
     <row r="226">
-      <c r="B226" s="5" t="n"/>
-      <c r="C226" s="5" t="n"/>
+      <c r="A226" s="5" t="n"/>
+      <c r="F226" s="5" t="n"/>
       <c r="K226" s="5" t="n"/>
     </row>
     <row r="227">
-      <c r="B227" s="5" t="n"/>
-      <c r="C227" s="5" t="n"/>
+      <c r="A227" s="5" t="n"/>
+      <c r="F227" s="5" t="n"/>
       <c r="K227" s="5" t="n"/>
     </row>
     <row r="228">
-      <c r="B228" s="5" t="n"/>
-      <c r="C228" s="5" t="n"/>
+      <c r="A228" s="5" t="n"/>
+      <c r="F228" s="5" t="n"/>
       <c r="K228" s="5" t="n"/>
     </row>
     <row r="229">
-      <c r="B229" s="5" t="n"/>
-      <c r="C229" s="5" t="n"/>
+      <c r="A229" s="5" t="n"/>
+      <c r="F229" s="5" t="n"/>
       <c r="K229" s="5" t="n"/>
     </row>
     <row r="230">
-      <c r="B230" s="5" t="n"/>
-      <c r="C230" s="5" t="n"/>
+      <c r="A230" s="5" t="n"/>
+      <c r="F230" s="5" t="n"/>
       <c r="K230" s="5" t="n"/>
     </row>
     <row r="231">
-      <c r="B231" s="5" t="n"/>
-      <c r="C231" s="5" t="n"/>
+      <c r="A231" s="5" t="n"/>
+      <c r="F231" s="5" t="n"/>
       <c r="K231" s="5" t="n"/>
     </row>
     <row r="232">
-      <c r="B232" s="5" t="n"/>
-      <c r="C232" s="5" t="n"/>
+      <c r="A232" s="5" t="n"/>
+      <c r="F232" s="5" t="n"/>
       <c r="K232" s="5" t="n"/>
     </row>
     <row r="233">
-      <c r="B233" s="5" t="n"/>
-      <c r="C233" s="5" t="n"/>
+      <c r="A233" s="5" t="n"/>
+      <c r="F233" s="5" t="n"/>
       <c r="K233" s="5" t="n"/>
     </row>
     <row r="234">
-      <c r="B234" s="5" t="n"/>
-      <c r="C234" s="5" t="n"/>
+      <c r="A234" s="5" t="n"/>
+      <c r="F234" s="5" t="n"/>
       <c r="K234" s="5" t="n"/>
     </row>
     <row r="235">
-      <c r="B235" s="5" t="n"/>
-      <c r="C235" s="5" t="n"/>
+      <c r="A235" s="5" t="n"/>
+      <c r="F235" s="5" t="n"/>
       <c r="K235" s="5" t="n"/>
     </row>
     <row r="236">
-      <c r="B236" s="5" t="n"/>
-      <c r="C236" s="5" t="n"/>
+      <c r="A236" s="5" t="n"/>
+      <c r="F236" s="5" t="n"/>
       <c r="K236" s="5" t="n"/>
     </row>
     <row r="237">
-      <c r="B237" s="5" t="n"/>
-      <c r="C237" s="5" t="n"/>
+      <c r="A237" s="5" t="n"/>
+      <c r="F237" s="5" t="n"/>
       <c r="K237" s="5" t="n"/>
     </row>
     <row r="238">
-      <c r="B238" s="5" t="n"/>
-      <c r="C238" s="5" t="n"/>
+      <c r="A238" s="5" t="n"/>
+      <c r="F238" s="5" t="n"/>
       <c r="K238" s="5" t="n"/>
     </row>
     <row r="239">
-      <c r="B239" s="5" t="n"/>
-      <c r="C239" s="5" t="n"/>
+      <c r="A239" s="5" t="n"/>
+      <c r="F239" s="5" t="n"/>
       <c r="K239" s="5" t="n"/>
     </row>
     <row r="240">
-      <c r="B240" s="5" t="n"/>
-      <c r="C240" s="5" t="n"/>
+      <c r="A240" s="5" t="n"/>
+      <c r="F240" s="5" t="n"/>
       <c r="K240" s="5" t="n"/>
     </row>
     <row r="241">
-      <c r="B241" s="5" t="n"/>
-      <c r="C241" s="5" t="n"/>
+      <c r="A241" s="5" t="n"/>
+      <c r="F241" s="5" t="n"/>
       <c r="K241" s="5" t="n"/>
     </row>
     <row r="242">
-      <c r="B242" s="5" t="n"/>
-      <c r="C242" s="5" t="n"/>
+      <c r="A242" s="5" t="n"/>
+      <c r="F242" s="5" t="n"/>
       <c r="K242" s="5" t="n"/>
     </row>
     <row r="243">
-      <c r="B243" s="5" t="n"/>
-      <c r="C243" s="5" t="n"/>
+      <c r="A243" s="5" t="n"/>
+      <c r="F243" s="5" t="n"/>
       <c r="K243" s="5" t="n"/>
     </row>
     <row r="244">
-      <c r="B244" s="5" t="n"/>
-      <c r="C244" s="5" t="n"/>
+      <c r="A244" s="5" t="n"/>
+      <c r="F244" s="5" t="n"/>
       <c r="K244" s="5" t="n"/>
     </row>
     <row r="245">
-      <c r="B245" s="5" t="n"/>
-      <c r="C245" s="5" t="n"/>
+      <c r="A245" s="5" t="n"/>
+      <c r="F245" s="5" t="n"/>
       <c r="K245" s="5" t="n"/>
     </row>
     <row r="246">
-      <c r="B246" s="5" t="n"/>
-      <c r="C246" s="5" t="n"/>
+      <c r="A246" s="5" t="n"/>
+      <c r="F246" s="5" t="n"/>
       <c r="K246" s="5" t="n"/>
     </row>
     <row r="247">
-      <c r="B247" s="5" t="n"/>
-      <c r="C247" s="5" t="n"/>
+      <c r="A247" s="5" t="n"/>
+      <c r="F247" s="5" t="n"/>
       <c r="K247" s="5" t="n"/>
     </row>
     <row r="248">
-      <c r="B248" s="5" t="n"/>
-      <c r="C248" s="5" t="n"/>
+      <c r="A248" s="5" t="n"/>
+      <c r="F248" s="5" t="n"/>
       <c r="K248" s="5" t="n"/>
     </row>
     <row r="249">
-      <c r="B249" s="5" t="n"/>
-      <c r="C249" s="5" t="n"/>
+      <c r="A249" s="5" t="n"/>
+      <c r="F249" s="5" t="n"/>
       <c r="K249" s="5" t="n"/>
     </row>
     <row r="250">
-      <c r="B250" s="5" t="n"/>
-      <c r="C250" s="5" t="n"/>
+      <c r="A250" s="5" t="n"/>
+      <c r="F250" s="5" t="n"/>
       <c r="K250" s="5" t="n"/>
     </row>
     <row r="251">
-      <c r="B251" s="5" t="n"/>
-      <c r="C251" s="5" t="n"/>
+      <c r="A251" s="5" t="n"/>
+      <c r="F251" s="5" t="n"/>
       <c r="K251" s="5" t="n"/>
     </row>
     <row r="252">
-      <c r="B252" s="5" t="n"/>
-      <c r="C252" s="5" t="n"/>
+      <c r="A252" s="5" t="n"/>
+      <c r="F252" s="5" t="n"/>
       <c r="K252" s="5" t="n"/>
     </row>
     <row r="253">
-      <c r="B253" s="5" t="n"/>
-      <c r="C253" s="5" t="n"/>
+      <c r="A253" s="5" t="n"/>
+      <c r="F253" s="5" t="n"/>
       <c r="K253" s="5" t="n"/>
     </row>
     <row r="254">
-      <c r="B254" s="5" t="n"/>
-      <c r="C254" s="5" t="n"/>
+      <c r="A254" s="5" t="n"/>
+      <c r="F254" s="5" t="n"/>
       <c r="K254" s="5" t="n"/>
     </row>
     <row r="255">
-      <c r="B255" s="5" t="n"/>
-      <c r="C255" s="5" t="n"/>
+      <c r="A255" s="5" t="n"/>
+      <c r="F255" s="5" t="n"/>
       <c r="K255" s="5" t="n"/>
     </row>
     <row r="256">
-      <c r="B256" s="5" t="n"/>
-      <c r="C256" s="5" t="n"/>
+      <c r="A256" s="5" t="n"/>
+      <c r="F256" s="5" t="n"/>
       <c r="K256" s="5" t="n"/>
     </row>
     <row r="257">
-      <c r="B257" s="5" t="n"/>
-      <c r="C257" s="5" t="n"/>
+      <c r="A257" s="5" t="n"/>
+      <c r="F257" s="5" t="n"/>
       <c r="K257" s="5" t="n"/>
     </row>
     <row r="258">
-      <c r="B258" s="5" t="n"/>
-      <c r="C258" s="5" t="n"/>
+      <c r="A258" s="5" t="n"/>
+      <c r="F258" s="5" t="n"/>
       <c r="K258" s="5" t="n"/>
     </row>
     <row r="259">
-      <c r="B259" s="5" t="n"/>
-      <c r="C259" s="5" t="n"/>
+      <c r="A259" s="5" t="n"/>
+      <c r="F259" s="5" t="n"/>
       <c r="K259" s="5" t="n"/>
     </row>
     <row r="260">
-      <c r="B260" s="5" t="n"/>
-      <c r="C260" s="5" t="n"/>
+      <c r="A260" s="5" t="n"/>
+      <c r="F260" s="5" t="n"/>
       <c r="K260" s="5" t="n"/>
     </row>
     <row r="261">
-      <c r="B261" s="5" t="n"/>
-      <c r="C261" s="5" t="n"/>
+      <c r="A261" s="5" t="n"/>
+      <c r="F261" s="5" t="n"/>
       <c r="K261" s="5" t="n"/>
     </row>
     <row r="262">
-      <c r="B262" s="5" t="n"/>
-      <c r="C262" s="5" t="n"/>
+      <c r="A262" s="5" t="n"/>
+      <c r="F262" s="5" t="n"/>
       <c r="K262" s="5" t="n"/>
     </row>
     <row r="263">
-      <c r="B263" s="5" t="n"/>
-      <c r="C263" s="5" t="n"/>
+      <c r="A263" s="5" t="n"/>
+      <c r="F263" s="5" t="n"/>
       <c r="K263" s="5" t="n"/>
     </row>
     <row r="264">
-      <c r="B264" s="5" t="n"/>
-      <c r="C264" s="5" t="n"/>
+      <c r="A264" s="5" t="n"/>
+      <c r="F264" s="5" t="n"/>
       <c r="K264" s="5" t="n"/>
     </row>
     <row r="265">
-      <c r="B265" s="5" t="n"/>
-      <c r="C265" s="5" t="n"/>
+      <c r="A265" s="5" t="n"/>
+      <c r="F265" s="5" t="n"/>
       <c r="K265" s="5" t="n"/>
     </row>
     <row r="266">
-      <c r="B266" s="5" t="n"/>
-      <c r="C266" s="5" t="n"/>
+      <c r="A266" s="5" t="n"/>
+      <c r="F266" s="5" t="n"/>
       <c r="K266" s="5" t="n"/>
     </row>
     <row r="267">
-      <c r="B267" s="5" t="n"/>
-      <c r="C267" s="5" t="n"/>
+      <c r="A267" s="5" t="n"/>
+      <c r="F267" s="5" t="n"/>
       <c r="K267" s="5" t="n"/>
     </row>
     <row r="268">
-      <c r="B268" s="5" t="n"/>
-      <c r="C268" s="5" t="n"/>
+      <c r="A268" s="5" t="n"/>
+      <c r="F268" s="5" t="n"/>
       <c r="K268" s="5" t="n"/>
     </row>
     <row r="269">
-      <c r="B269" s="5" t="n"/>
-      <c r="C269" s="5" t="n"/>
+      <c r="A269" s="5" t="n"/>
+      <c r="F269" s="5" t="n"/>
       <c r="K269" s="5" t="n"/>
     </row>
     <row r="270">
-      <c r="B270" s="5" t="n"/>
-      <c r="C270" s="5" t="n"/>
+      <c r="A270" s="5" t="n"/>
+      <c r="F270" s="5" t="n"/>
       <c r="K270" s="5" t="n"/>
     </row>
     <row r="271">
-      <c r="B271" s="5" t="n"/>
-      <c r="C271" s="5" t="n"/>
+      <c r="A271" s="5" t="n"/>
+      <c r="F271" s="5" t="n"/>
       <c r="K271" s="5" t="n"/>
     </row>
     <row r="272">
-      <c r="B272" s="5" t="n"/>
-      <c r="C272" s="5" t="n"/>
+      <c r="A272" s="5" t="n"/>
+      <c r="F272" s="5" t="n"/>
       <c r="K272" s="5" t="n"/>
     </row>
     <row r="273">
-      <c r="B273" s="5" t="n"/>
-      <c r="C273" s="5" t="n"/>
+      <c r="A273" s="5" t="n"/>
+      <c r="F273" s="5" t="n"/>
       <c r="K273" s="5" t="n"/>
     </row>
     <row r="274">
-      <c r="B274" s="5" t="n"/>
-      <c r="C274" s="5" t="n"/>
+      <c r="A274" s="5" t="n"/>
+      <c r="F274" s="5" t="n"/>
       <c r="K274" s="5" t="n"/>
     </row>
     <row r="275">
-      <c r="B275" s="5" t="n"/>
-      <c r="C275" s="5" t="n"/>
+      <c r="A275" s="5" t="n"/>
+      <c r="F275" s="5" t="n"/>
       <c r="K275" s="5" t="n"/>
     </row>
     <row r="276">
-      <c r="B276" s="5" t="n"/>
-      <c r="C276" s="5" t="n"/>
+      <c r="A276" s="5" t="n"/>
+      <c r="F276" s="5" t="n"/>
       <c r="K276" s="5" t="n"/>
     </row>
     <row r="277">
-      <c r="B277" s="5" t="n"/>
-      <c r="C277" s="5" t="n"/>
+      <c r="A277" s="5" t="n"/>
+      <c r="F277" s="5" t="n"/>
       <c r="K277" s="5" t="n"/>
     </row>
     <row r="278">
-      <c r="B278" s="5" t="n"/>
-      <c r="C278" s="5" t="n"/>
+      <c r="A278" s="5" t="n"/>
+      <c r="F278" s="5" t="n"/>
       <c r="K278" s="5" t="n"/>
     </row>
     <row r="279">
-      <c r="B279" s="5" t="n"/>
-      <c r="C279" s="5" t="n"/>
+      <c r="A279" s="5" t="n"/>
+      <c r="F279" s="5" t="n"/>
       <c r="K279" s="5" t="n"/>
     </row>
     <row r="280">
-      <c r="B280" s="5" t="n"/>
-      <c r="C280" s="5" t="n"/>
+      <c r="A280" s="5" t="n"/>
+      <c r="F280" s="5" t="n"/>
       <c r="K280" s="5" t="n"/>
     </row>
     <row r="281">
-      <c r="B281" s="5" t="n"/>
-      <c r="C281" s="5" t="n"/>
+      <c r="A281" s="5" t="n"/>
+      <c r="F281" s="5" t="n"/>
       <c r="K281" s="5" t="n"/>
     </row>
     <row r="282">
-      <c r="B282" s="5" t="n"/>
-      <c r="C282" s="5" t="n"/>
+      <c r="A282" s="5" t="n"/>
+      <c r="F282" s="5" t="n"/>
       <c r="K282" s="5" t="n"/>
     </row>
     <row r="283">
-      <c r="B283" s="5" t="n"/>
-      <c r="C283" s="5" t="n"/>
+      <c r="A283" s="5" t="n"/>
+      <c r="F283" s="5" t="n"/>
       <c r="K283" s="5" t="n"/>
     </row>
     <row r="284">
-      <c r="B284" s="5" t="n"/>
-      <c r="C284" s="5" t="n"/>
+      <c r="A284" s="5" t="n"/>
+      <c r="F284" s="5" t="n"/>
       <c r="K284" s="5" t="n"/>
     </row>
     <row r="285">
-      <c r="B285" s="5" t="n"/>
-      <c r="C285" s="5" t="n"/>
+      <c r="A285" s="5" t="n"/>
+      <c r="F285" s="5" t="n"/>
       <c r="K285" s="5" t="n"/>
     </row>
     <row r="286">
-      <c r="B286" s="5" t="n"/>
-      <c r="C286" s="5" t="n"/>
+      <c r="A286" s="5" t="n"/>
+      <c r="F286" s="5" t="n"/>
       <c r="K286" s="5" t="n"/>
     </row>
     <row r="287">
-      <c r="B287" s="5" t="n"/>
-      <c r="C287" s="5" t="n"/>
+      <c r="A287" s="5" t="n"/>
+      <c r="F287" s="5" t="n"/>
       <c r="K287" s="5" t="n"/>
     </row>
     <row r="288">
-      <c r="B288" s="5" t="n"/>
-      <c r="C288" s="5" t="n"/>
+      <c r="A288" s="5" t="n"/>
+      <c r="F288" s="5" t="n"/>
       <c r="K288" s="5" t="n"/>
     </row>
     <row r="289">
-      <c r="B289" s="5" t="n"/>
-      <c r="C289" s="5" t="n"/>
+      <c r="A289" s="5" t="n"/>
+      <c r="F289" s="5" t="n"/>
       <c r="K289" s="5" t="n"/>
     </row>
     <row r="290">
-      <c r="B290" s="5" t="n"/>
-      <c r="C290" s="5" t="n"/>
+      <c r="A290" s="5" t="n"/>
+      <c r="F290" s="5" t="n"/>
       <c r="K290" s="5" t="n"/>
     </row>
     <row r="291">
-      <c r="B291" s="5" t="n"/>
-      <c r="C291" s="5" t="n"/>
+      <c r="A291" s="5" t="n"/>
+      <c r="F291" s="5" t="n"/>
       <c r="K291" s="5" t="n"/>
     </row>
     <row r="292">
-      <c r="B292" s="5" t="n"/>
-      <c r="C292" s="5" t="n"/>
+      <c r="A292" s="5" t="n"/>
+      <c r="F292" s="5" t="n"/>
       <c r="K292" s="5" t="n"/>
     </row>
     <row r="293">
-      <c r="B293" s="5" t="n"/>
-      <c r="C293" s="5" t="n"/>
+      <c r="A293" s="5" t="n"/>
+      <c r="F293" s="5" t="n"/>
       <c r="K293" s="5" t="n"/>
     </row>
     <row r="294">
-      <c r="B294" s="5" t="n"/>
-      <c r="C294" s="5" t="n"/>
+      <c r="A294" s="5" t="n"/>
+      <c r="F294" s="5" t="n"/>
       <c r="K294" s="5" t="n"/>
     </row>
     <row r="295">
-      <c r="B295" s="5" t="n"/>
-      <c r="C295" s="5" t="n"/>
+      <c r="A295" s="5" t="n"/>
+      <c r="F295" s="5" t="n"/>
       <c r="K295" s="5" t="n"/>
     </row>
     <row r="296">
-      <c r="B296" s="5" t="n"/>
-      <c r="C296" s="5" t="n"/>
+      <c r="A296" s="5" t="n"/>
+      <c r="F296" s="5" t="n"/>
       <c r="K296" s="5" t="n"/>
     </row>
     <row r="297">
-      <c r="B297" s="5" t="n"/>
-      <c r="C297" s="5" t="n"/>
+      <c r="A297" s="5" t="n"/>
+      <c r="F297" s="5" t="n"/>
       <c r="K297" s="5" t="n"/>
     </row>
     <row r="298">
-      <c r="B298" s="5" t="n"/>
-      <c r="C298" s="5" t="n"/>
+      <c r="A298" s="5" t="n"/>
+      <c r="F298" s="5" t="n"/>
       <c r="K298" s="5" t="n"/>
     </row>
     <row r="299">
-      <c r="B299" s="5" t="n"/>
-      <c r="C299" s="5" t="n"/>
+      <c r="A299" s="5" t="n"/>
+      <c r="F299" s="5" t="n"/>
       <c r="K299" s="5" t="n"/>
     </row>
     <row r="300">
-      <c r="B300" s="5" t="n"/>
-      <c r="C300" s="5" t="n"/>
+      <c r="A300" s="5" t="n"/>
+      <c r="F300" s="5" t="n"/>
       <c r="K300" s="5" t="n"/>
     </row>
     <row r="301">
-      <c r="B301" s="5" t="n"/>
-      <c r="C301" s="5" t="n"/>
+      <c r="A301" s="5" t="n"/>
+      <c r="F301" s="5" t="n"/>
       <c r="K301" s="5" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="4">
-    <dataValidation sqref="A2:A301" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="ערך לא תקין" error="יש לבחור ערך מהרשימה" type="list">
+    <dataValidation sqref="C2:C301" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="ערך לא תקין" error="יש לבחור ערך מהרשימה" type="list">
       <formula1>='רשימות'!$A$1:$A$5</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D301" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="ערך לא תקין" error="יש לבחור ערך מהרשימה" type="list">
+    <dataValidation sqref="B2:B301" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="ערך לא תקין" error="יש לבחור ערך מהרשימה" type="list">
       <formula1>='רשימות'!$B$1:$B$5</formula1>
     </dataValidation>
-    <dataValidation sqref="E2:E301" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="ערך לא תקין" error="יש לבחור ערך מהרשימה" type="list">
+    <dataValidation sqref="D2:D301" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="ערך לא תקין" error="יש לבחור ערך מהרשימה" type="list">
       <formula1>='רשימות'!$C$1:$C$6</formula1>
     </dataValidation>
-    <dataValidation sqref="N2:N301" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="ערך לא תקין" error="יש לבחור ערך מהרשימה" type="list">
+    <dataValidation sqref="M2:M301" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="ערך לא תקין" error="יש לבחור ערך מהרשימה" type="list">
       <formula1>='רשימות'!$D$1:$D$6</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
fix: vehicle type is required again; no "אחר" fallback
Per Tamir: vehicle type is a required field. Asterisk + validation that blocks
with a message, required in Excel import and template; the "אחר" default is gone.
Shtifomat stays optional (empty is sent as "לא").

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/order-template.xlsx
+++ b/order-template.xlsx
@@ -478,7 +478,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>3. שטיפומט: «לא», או מספר השטיפות בחודש (1 עד 5). ריק = «לא». סוג רכב ריק = «אחר».</t>
+          <t>3. שטיפומט: «לא», או מספר השטיפות בחודש (1 עד 5). ריק = «לא».</t>
         </is>
       </c>
     </row>
@@ -573,9 +573,9 @@
           <t>סוג אמצעי תדלוק *</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
-        <is>
-          <t>סוג הרכב</t>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>סוג הרכב *</t>
         </is>
       </c>
       <c r="E1" s="4" t="inlineStr">

</xml_diff>